<commit_message>
Updated on 10-30-2023 at 00:07
</commit_message>
<xml_diff>
--- a/output/accuracy_cubic.xlsx
+++ b/output/accuracy_cubic.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N27"/>
+  <dimension ref="A1:N17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -474,43 +474,43 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>5</v>
+        <v>45</v>
       </c>
       <c r="C2" t="n">
-        <v>0.0028902</v>
+        <v>0.032975</v>
       </c>
       <c r="D2" t="n">
-        <v>0.39</v>
+        <v>4.31</v>
       </c>
       <c r="E2" t="n">
-        <v>1.13</v>
+        <v>0.26</v>
       </c>
       <c r="F2" t="n">
-        <v>5.81</v>
+        <v>1.91</v>
       </c>
       <c r="G2" t="n">
-        <v>21.29</v>
+        <v>2.73</v>
       </c>
       <c r="H2" t="n">
-        <v>42.15</v>
+        <v>1.42</v>
       </c>
       <c r="I2" t="n">
-        <v>68.61</v>
+        <v>0.55</v>
       </c>
       <c r="J2" t="n">
-        <v>100.42</v>
+        <v>2.95</v>
       </c>
       <c r="K2" t="n">
-        <v>142.17</v>
+        <v>2.4</v>
       </c>
       <c r="L2" t="n">
-        <v>193.58</v>
+        <v>3.03</v>
       </c>
       <c r="M2" t="n">
-        <v>255.32</v>
+        <v>0.02</v>
       </c>
       <c r="N2" t="n">
-        <v>83.09</v>
+        <v>1.96</v>
       </c>
     </row>
     <row r="3">
@@ -518,43 +518,43 @@
         <v>1</v>
       </c>
       <c r="B3" t="n">
-        <v>6</v>
+        <v>46</v>
       </c>
       <c r="C3" t="n">
-        <v>0.0043706</v>
+        <v>0.038934</v>
       </c>
       <c r="D3" t="n">
-        <v>2.69</v>
+        <v>4.34</v>
       </c>
       <c r="E3" t="n">
-        <v>9.42</v>
+        <v>0.37</v>
       </c>
       <c r="F3" t="n">
-        <v>18.5</v>
+        <v>1.65</v>
       </c>
       <c r="G3" t="n">
-        <v>22.42</v>
+        <v>2.26</v>
       </c>
       <c r="H3" t="n">
-        <v>27.73</v>
+        <v>2.14</v>
       </c>
       <c r="I3" t="n">
-        <v>34.19</v>
+        <v>0.51</v>
       </c>
       <c r="J3" t="n">
-        <v>51.61</v>
+        <v>1.45</v>
       </c>
       <c r="K3" t="n">
-        <v>71.31</v>
+        <v>0.43</v>
       </c>
       <c r="L3" t="n">
-        <v>92.25</v>
+        <v>5.43</v>
       </c>
       <c r="M3" t="n">
-        <v>116.48</v>
+        <v>3.12</v>
       </c>
       <c r="N3" t="n">
-        <v>44.66</v>
+        <v>2.17</v>
       </c>
     </row>
     <row r="4">
@@ -562,43 +562,43 @@
         <v>2</v>
       </c>
       <c r="B4" t="n">
-        <v>7</v>
+        <v>47</v>
       </c>
       <c r="C4" t="n">
-        <v>2.6973e-05</v>
+        <v>0.04607</v>
       </c>
       <c r="D4" t="n">
-        <v>0.53</v>
+        <v>4.35</v>
       </c>
       <c r="E4" t="n">
-        <v>3.91</v>
+        <v>0.41</v>
       </c>
       <c r="F4" t="n">
-        <v>8.199999999999999</v>
+        <v>1.58</v>
       </c>
       <c r="G4" t="n">
-        <v>6.63</v>
+        <v>2.14</v>
       </c>
       <c r="H4" t="n">
-        <v>5.5</v>
+        <v>2.32</v>
       </c>
       <c r="I4" t="n">
-        <v>4.71</v>
+        <v>0.76</v>
       </c>
       <c r="J4" t="n">
-        <v>11.63</v>
+        <v>1.11</v>
       </c>
       <c r="K4" t="n">
-        <v>19.15</v>
+        <v>0</v>
       </c>
       <c r="L4" t="n">
-        <v>26.7</v>
+        <v>5.94</v>
       </c>
       <c r="M4" t="n">
-        <v>35.81</v>
+        <v>3.76</v>
       </c>
       <c r="N4" t="n">
-        <v>12.28</v>
+        <v>2.24</v>
       </c>
     </row>
     <row r="5">
@@ -606,43 +606,43 @@
         <v>3</v>
       </c>
       <c r="B5" t="n">
-        <v>8</v>
+        <v>48</v>
       </c>
       <c r="C5" t="n">
-        <v>0.00016596</v>
+        <v>0.054777</v>
       </c>
       <c r="D5" t="n">
-        <v>0.91</v>
+        <v>4.36</v>
       </c>
       <c r="E5" t="n">
-        <v>4.62</v>
+        <v>0.41</v>
       </c>
       <c r="F5" t="n">
-        <v>9.140000000000001</v>
+        <v>1.58</v>
       </c>
       <c r="G5" t="n">
-        <v>7.55</v>
+        <v>2.15</v>
       </c>
       <c r="H5" t="n">
-        <v>6.13</v>
+        <v>2.29</v>
       </c>
       <c r="I5" t="n">
-        <v>4.77</v>
+        <v>0.72</v>
       </c>
       <c r="J5" t="n">
-        <v>10.75</v>
+        <v>1.17</v>
       </c>
       <c r="K5" t="n">
-        <v>16.87</v>
+        <v>0.09</v>
       </c>
       <c r="L5" t="n">
-        <v>22.55</v>
+        <v>5.83</v>
       </c>
       <c r="M5" t="n">
-        <v>29.25</v>
+        <v>3.62</v>
       </c>
       <c r="N5" t="n">
-        <v>11.25</v>
+        <v>2.22</v>
       </c>
     </row>
     <row r="6">
@@ -650,43 +650,43 @@
         <v>4</v>
       </c>
       <c r="B6" t="n">
-        <v>9</v>
+        <v>49</v>
       </c>
       <c r="C6" t="n">
-        <v>0.00027254</v>
+        <v>0.008087199999999999</v>
       </c>
       <c r="D6" t="n">
-        <v>0.63</v>
+        <v>4.39</v>
       </c>
       <c r="E6" t="n">
-        <v>3.8</v>
+        <v>0.27</v>
       </c>
       <c r="F6" t="n">
-        <v>7.43</v>
+        <v>2.1</v>
       </c>
       <c r="G6" t="n">
-        <v>4.67</v>
+        <v>3.27</v>
       </c>
       <c r="H6" t="n">
-        <v>1.76</v>
+        <v>0.44</v>
       </c>
       <c r="I6" t="n">
-        <v>1.39</v>
+        <v>2.18</v>
       </c>
       <c r="J6" t="n">
-        <v>1.95</v>
+        <v>5.39</v>
       </c>
       <c r="K6" t="n">
-        <v>4.86</v>
+        <v>5.77</v>
       </c>
       <c r="L6" t="n">
-        <v>6.85</v>
+        <v>1.19</v>
       </c>
       <c r="M6" t="n">
-        <v>9.24</v>
+        <v>5.56</v>
       </c>
       <c r="N6" t="n">
-        <v>4.26</v>
+        <v>3.06</v>
       </c>
     </row>
     <row r="7">
@@ -694,43 +694,43 @@
         <v>5</v>
       </c>
       <c r="B7" t="n">
-        <v>10</v>
+        <v>50</v>
       </c>
       <c r="C7" t="n">
-        <v>0.0006367</v>
+        <v>0.0081095</v>
       </c>
       <c r="D7" t="n">
-        <v>0.55</v>
+        <v>4.36</v>
       </c>
       <c r="E7" t="n">
-        <v>3.71</v>
+        <v>0.22</v>
       </c>
       <c r="F7" t="n">
-        <v>7.43</v>
+        <v>2.19</v>
       </c>
       <c r="G7" t="n">
-        <v>4.92</v>
+        <v>3.39</v>
       </c>
       <c r="H7" t="n">
-        <v>2.41</v>
+        <v>0.29</v>
       </c>
       <c r="I7" t="n">
-        <v>0.19</v>
+        <v>2.36</v>
       </c>
       <c r="J7" t="n">
-        <v>3.99</v>
+        <v>5.62</v>
       </c>
       <c r="K7" t="n">
-        <v>8.01</v>
+        <v>6.04</v>
       </c>
       <c r="L7" t="n">
-        <v>11.37</v>
+        <v>1.49</v>
       </c>
       <c r="M7" t="n">
-        <v>15.42</v>
+        <v>5.92</v>
       </c>
       <c r="N7" t="n">
-        <v>5.8</v>
+        <v>3.19</v>
       </c>
     </row>
     <row r="8">
@@ -738,43 +738,43 @@
         <v>6</v>
       </c>
       <c r="B8" t="n">
-        <v>11</v>
+        <v>51</v>
       </c>
       <c r="C8" t="n">
-        <v>0.00089059</v>
+        <v>0.0081481</v>
       </c>
       <c r="D8" t="n">
-        <v>0.15</v>
+        <v>4.39</v>
       </c>
       <c r="E8" t="n">
-        <v>2.56</v>
+        <v>0.29</v>
       </c>
       <c r="F8" t="n">
-        <v>5.08</v>
+        <v>2.08</v>
       </c>
       <c r="G8" t="n">
-        <v>1.02</v>
+        <v>3.24</v>
       </c>
       <c r="H8" t="n">
-        <v>3.44</v>
+        <v>0.48</v>
       </c>
       <c r="I8" t="n">
-        <v>8.369999999999999</v>
+        <v>2.13</v>
       </c>
       <c r="J8" t="n">
-        <v>7.63</v>
+        <v>5.33</v>
       </c>
       <c r="K8" t="n">
-        <v>7.76</v>
+        <v>5.7</v>
       </c>
       <c r="L8" t="n">
-        <v>9.17</v>
+        <v>1.11</v>
       </c>
       <c r="M8" t="n">
-        <v>10.67</v>
+        <v>5.46</v>
       </c>
       <c r="N8" t="n">
-        <v>5.58</v>
+        <v>3.02</v>
       </c>
     </row>
     <row r="9">
@@ -782,43 +782,43 @@
         <v>7</v>
       </c>
       <c r="B9" t="n">
-        <v>12</v>
+        <v>52</v>
       </c>
       <c r="C9" t="n">
-        <v>0.00089061</v>
+        <v>0.008276499999999999</v>
       </c>
       <c r="D9" t="n">
-        <v>0.14</v>
+        <v>4.45</v>
       </c>
       <c r="E9" t="n">
-        <v>2.54</v>
+        <v>0.41</v>
       </c>
       <c r="F9" t="n">
-        <v>5.04</v>
+        <v>1.89</v>
       </c>
       <c r="G9" t="n">
-        <v>0.97</v>
+        <v>2.97</v>
       </c>
       <c r="H9" t="n">
-        <v>3.52</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="I9" t="n">
-        <v>8.48</v>
+        <v>1.7</v>
       </c>
       <c r="J9" t="n">
-        <v>7.78</v>
+        <v>4.81</v>
       </c>
       <c r="K9" t="n">
-        <v>7.97</v>
+        <v>5.08</v>
       </c>
       <c r="L9" t="n">
-        <v>9.43</v>
+        <v>0.43</v>
       </c>
       <c r="M9" t="n">
-        <v>11</v>
+        <v>4.65</v>
       </c>
       <c r="N9" t="n">
-        <v>5.69</v>
+        <v>2.72</v>
       </c>
     </row>
     <row r="10">
@@ -826,43 +826,43 @@
         <v>8</v>
       </c>
       <c r="B10" t="n">
-        <v>13</v>
+        <v>53</v>
       </c>
       <c r="C10" t="n">
-        <v>0.0010644</v>
+        <v>0.008313900000000001</v>
       </c>
       <c r="D10" t="n">
-        <v>0.02</v>
+        <v>4.42</v>
       </c>
       <c r="E10" t="n">
-        <v>2.1</v>
+        <v>0.34</v>
       </c>
       <c r="F10" t="n">
-        <v>4.19</v>
+        <v>2</v>
       </c>
       <c r="G10" t="n">
-        <v>0.36</v>
+        <v>3.12</v>
       </c>
       <c r="H10" t="n">
-        <v>5.43</v>
+        <v>0.63</v>
       </c>
       <c r="I10" t="n">
-        <v>11.07</v>
+        <v>1.93</v>
       </c>
       <c r="J10" t="n">
-        <v>11.35</v>
+        <v>5.09</v>
       </c>
       <c r="K10" t="n">
-        <v>12.69</v>
+        <v>5.41</v>
       </c>
       <c r="L10" t="n">
-        <v>15.45</v>
+        <v>0.79</v>
       </c>
       <c r="M10" t="n">
-        <v>18.49</v>
+        <v>5.08</v>
       </c>
       <c r="N10" t="n">
-        <v>8.109999999999999</v>
+        <v>2.88</v>
       </c>
     </row>
     <row r="11">
@@ -870,43 +870,43 @@
         <v>9</v>
       </c>
       <c r="B11" t="n">
-        <v>14</v>
+        <v>54</v>
       </c>
       <c r="C11" t="n">
-        <v>0.00031342</v>
+        <v>0.008314999999999999</v>
       </c>
       <c r="D11" t="n">
-        <v>0.4</v>
+        <v>4.42</v>
       </c>
       <c r="E11" t="n">
-        <v>3.17</v>
+        <v>0.35</v>
       </c>
       <c r="F11" t="n">
-        <v>6.19</v>
+        <v>1.98</v>
       </c>
       <c r="G11" t="n">
-        <v>2.72</v>
+        <v>3.09</v>
       </c>
       <c r="H11" t="n">
-        <v>1.08</v>
+        <v>0.66</v>
       </c>
       <c r="I11" t="n">
-        <v>5.26</v>
+        <v>1.89</v>
       </c>
       <c r="J11" t="n">
-        <v>3.43</v>
+        <v>5.04</v>
       </c>
       <c r="K11" t="n">
-        <v>2.31</v>
+        <v>5.35</v>
       </c>
       <c r="L11" t="n">
-        <v>2.34</v>
+        <v>0.73</v>
       </c>
       <c r="M11" t="n">
-        <v>2.29</v>
+        <v>5.01</v>
       </c>
       <c r="N11" t="n">
-        <v>2.92</v>
+        <v>2.85</v>
       </c>
     </row>
     <row r="12">
@@ -914,43 +914,43 @@
         <v>10</v>
       </c>
       <c r="B12" t="n">
-        <v>15</v>
+        <v>55</v>
       </c>
       <c r="C12" t="n">
-        <v>0.00064893</v>
+        <v>0.0083599</v>
       </c>
       <c r="D12" t="n">
-        <v>0.37</v>
+        <v>4.39</v>
       </c>
       <c r="E12" t="n">
-        <v>3.1</v>
+        <v>0.28</v>
       </c>
       <c r="F12" t="n">
-        <v>6.04</v>
+        <v>2.09</v>
       </c>
       <c r="G12" t="n">
-        <v>2.44</v>
+        <v>3.25</v>
       </c>
       <c r="H12" t="n">
-        <v>1.51</v>
+        <v>0.47</v>
       </c>
       <c r="I12" t="n">
-        <v>5.88</v>
+        <v>2.14</v>
       </c>
       <c r="J12" t="n">
-        <v>4.34</v>
+        <v>5.34</v>
       </c>
       <c r="K12" t="n">
-        <v>3.56</v>
+        <v>5.71</v>
       </c>
       <c r="L12" t="n">
-        <v>3.99</v>
+        <v>1.12</v>
       </c>
       <c r="M12" t="n">
-        <v>4.4</v>
+        <v>5.48</v>
       </c>
       <c r="N12" t="n">
-        <v>3.56</v>
+        <v>3.03</v>
       </c>
     </row>
     <row r="13">
@@ -958,43 +958,43 @@
         <v>11</v>
       </c>
       <c r="B13" t="n">
-        <v>16</v>
+        <v>56</v>
       </c>
       <c r="C13" t="n">
-        <v>0.001376</v>
+        <v>0.0075223</v>
       </c>
       <c r="D13" t="n">
-        <v>0.32</v>
+        <v>4.25</v>
       </c>
       <c r="E13" t="n">
-        <v>2.97</v>
+        <v>0.02</v>
       </c>
       <c r="F13" t="n">
-        <v>5.8</v>
+        <v>2.57</v>
       </c>
       <c r="G13" t="n">
-        <v>2.09</v>
+        <v>3.92</v>
       </c>
       <c r="H13" t="n">
-        <v>1.98</v>
+        <v>0.36</v>
       </c>
       <c r="I13" t="n">
-        <v>6.5</v>
+        <v>3.18</v>
       </c>
       <c r="J13" t="n">
-        <v>5.15</v>
+        <v>6.62</v>
       </c>
       <c r="K13" t="n">
-        <v>4.6</v>
+        <v>7.21</v>
       </c>
       <c r="L13" t="n">
-        <v>5.27</v>
+        <v>2.76</v>
       </c>
       <c r="M13" t="n">
-        <v>5.95</v>
+        <v>7.41</v>
       </c>
       <c r="N13" t="n">
-        <v>4.06</v>
+        <v>3.83</v>
       </c>
     </row>
     <row r="14">
@@ -1002,43 +1002,43 @@
         <v>12</v>
       </c>
       <c r="B14" t="n">
-        <v>17</v>
+        <v>57</v>
       </c>
       <c r="C14" t="n">
-        <v>0.0034799</v>
+        <v>0.0075373</v>
       </c>
       <c r="D14" t="n">
-        <v>0.36</v>
+        <v>4.23</v>
       </c>
       <c r="E14" t="n">
-        <v>3.07</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="F14" t="n">
-        <v>5.98</v>
+        <v>2.64</v>
       </c>
       <c r="G14" t="n">
-        <v>2.36</v>
+        <v>4.01</v>
       </c>
       <c r="H14" t="n">
-        <v>1.61</v>
+        <v>0.47</v>
       </c>
       <c r="I14" t="n">
-        <v>6.01</v>
+        <v>3.32</v>
       </c>
       <c r="J14" t="n">
-        <v>4.51</v>
+        <v>6.8</v>
       </c>
       <c r="K14" t="n">
-        <v>3.78</v>
+        <v>7.41</v>
       </c>
       <c r="L14" t="n">
-        <v>4.25</v>
+        <v>2.99</v>
       </c>
       <c r="M14" t="n">
-        <v>4.71</v>
+        <v>7.68</v>
       </c>
       <c r="N14" t="n">
-        <v>3.67</v>
+        <v>3.96</v>
       </c>
     </row>
     <row r="15">
@@ -1046,43 +1046,43 @@
         <v>13</v>
       </c>
       <c r="B15" t="n">
-        <v>18</v>
+        <v>58</v>
       </c>
       <c r="C15" t="n">
-        <v>0.0064666</v>
+        <v>0.0078018</v>
       </c>
       <c r="D15" t="n">
-        <v>0.34</v>
+        <v>4.15</v>
       </c>
       <c r="E15" t="n">
-        <v>2.98</v>
+        <v>0.23</v>
       </c>
       <c r="F15" t="n">
-        <v>5.78</v>
+        <v>2.9</v>
       </c>
       <c r="G15" t="n">
-        <v>1.99</v>
+        <v>4.38</v>
       </c>
       <c r="H15" t="n">
-        <v>2.2</v>
+        <v>0.93</v>
       </c>
       <c r="I15" t="n">
-        <v>6.86</v>
+        <v>3.89</v>
       </c>
       <c r="J15" t="n">
-        <v>5.74</v>
+        <v>7.51</v>
       </c>
       <c r="K15" t="n">
-        <v>5.48</v>
+        <v>8.25</v>
       </c>
       <c r="L15" t="n">
-        <v>6.49</v>
+        <v>3.91</v>
       </c>
       <c r="M15" t="n">
-        <v>7.58</v>
+        <v>8.77</v>
       </c>
       <c r="N15" t="n">
-        <v>4.54</v>
+        <v>4.49</v>
       </c>
     </row>
     <row r="16">
@@ -1090,43 +1090,43 @@
         <v>14</v>
       </c>
       <c r="B16" t="n">
-        <v>19</v>
+        <v>59</v>
       </c>
       <c r="C16" t="n">
-        <v>0.008151200000000001</v>
+        <v>0.008195300000000001</v>
       </c>
       <c r="D16" t="n">
-        <v>0.29</v>
+        <v>4.06</v>
       </c>
       <c r="E16" t="n">
-        <v>2.72</v>
+        <v>0.43</v>
       </c>
       <c r="F16" t="n">
-        <v>5.08</v>
+        <v>3.22</v>
       </c>
       <c r="G16" t="n">
-        <v>0.65</v>
+        <v>4.82</v>
       </c>
       <c r="H16" t="n">
-        <v>4.43</v>
+        <v>1.47</v>
       </c>
       <c r="I16" t="n">
-        <v>10.21</v>
+        <v>4.58</v>
       </c>
       <c r="J16" t="n">
-        <v>10.76</v>
+        <v>8.359999999999999</v>
       </c>
       <c r="K16" t="n">
-        <v>12.59</v>
+        <v>9.24</v>
       </c>
       <c r="L16" t="n">
-        <v>16.06</v>
+        <v>5</v>
       </c>
       <c r="M16" t="n">
-        <v>20.08</v>
+        <v>10.07</v>
       </c>
       <c r="N16" t="n">
-        <v>8.289999999999999</v>
+        <v>5.12</v>
       </c>
     </row>
     <row r="17">
@@ -1134,483 +1134,43 @@
         <v>15</v>
       </c>
       <c r="B17" t="n">
-        <v>20</v>
+        <v>60</v>
       </c>
       <c r="C17" t="n">
-        <v>0.0085764</v>
+        <v>0.0084901</v>
       </c>
       <c r="D17" t="n">
-        <v>0.27</v>
+        <v>3.98</v>
       </c>
       <c r="E17" t="n">
-        <v>2.66</v>
+        <v>0.6</v>
       </c>
       <c r="F17" t="n">
-        <v>4.95</v>
+        <v>3.49</v>
       </c>
       <c r="G17" t="n">
-        <v>0.44</v>
+        <v>5.18</v>
       </c>
       <c r="H17" t="n">
-        <v>4.72</v>
+        <v>1.93</v>
       </c>
       <c r="I17" t="n">
-        <v>10.62</v>
+        <v>5.16</v>
       </c>
       <c r="J17" t="n">
-        <v>11.33</v>
+        <v>9.07</v>
       </c>
       <c r="K17" t="n">
-        <v>13.35</v>
+        <v>10.08</v>
       </c>
       <c r="L17" t="n">
-        <v>17.03</v>
+        <v>5.92</v>
       </c>
       <c r="M17" t="n">
-        <v>21.29</v>
+        <v>11.15</v>
       </c>
       <c r="N17" t="n">
-        <v>8.67</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="1" t="n">
-        <v>16</v>
-      </c>
-      <c r="B18" t="n">
-        <v>21</v>
-      </c>
-      <c r="C18" t="n">
-        <v>0.0024966</v>
-      </c>
-      <c r="D18" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="E18" t="n">
-        <v>2.63</v>
-      </c>
-      <c r="F18" t="n">
-        <v>4.92</v>
-      </c>
-      <c r="G18" t="n">
-        <v>0.42</v>
-      </c>
-      <c r="H18" t="n">
-        <v>4.73</v>
-      </c>
-      <c r="I18" t="n">
-        <v>10.6</v>
-      </c>
-      <c r="J18" t="n">
-        <v>11.27</v>
-      </c>
-      <c r="K18" t="n">
-        <v>13.24</v>
-      </c>
-      <c r="L18" t="n">
-        <v>16.87</v>
-      </c>
-      <c r="M18" t="n">
-        <v>21.05</v>
-      </c>
-      <c r="N18" t="n">
-        <v>8.6</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="1" t="n">
-        <v>17</v>
-      </c>
-      <c r="B19" t="n">
-        <v>22</v>
-      </c>
-      <c r="C19" t="n">
-        <v>0.0043649</v>
-      </c>
-      <c r="D19" t="n">
-        <v>0.29</v>
-      </c>
-      <c r="E19" t="n">
-        <v>2.74</v>
-      </c>
-      <c r="F19" t="n">
-        <v>5.15</v>
-      </c>
-      <c r="G19" t="n">
-        <v>0.78</v>
-      </c>
-      <c r="H19" t="n">
-        <v>4.21</v>
-      </c>
-      <c r="I19" t="n">
-        <v>9.9</v>
-      </c>
-      <c r="J19" t="n">
-        <v>10.3</v>
-      </c>
-      <c r="K19" t="n">
-        <v>11.96</v>
-      </c>
-      <c r="L19" t="n">
-        <v>15.24</v>
-      </c>
-      <c r="M19" t="n">
-        <v>19.02</v>
-      </c>
-      <c r="N19" t="n">
-        <v>7.96</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="1" t="n">
-        <v>18</v>
-      </c>
-      <c r="B20" t="n">
-        <v>23</v>
-      </c>
-      <c r="C20" t="n">
-        <v>0.0059763</v>
-      </c>
-      <c r="D20" t="n">
-        <v>0.27</v>
-      </c>
-      <c r="E20" t="n">
-        <v>2.7</v>
-      </c>
-      <c r="F20" t="n">
-        <v>5.08</v>
-      </c>
-      <c r="G20" t="n">
-        <v>0.68</v>
-      </c>
-      <c r="H20" t="n">
-        <v>4.34</v>
-      </c>
-      <c r="I20" t="n">
-        <v>10.06</v>
-      </c>
-      <c r="J20" t="n">
-        <v>10.51</v>
-      </c>
-      <c r="K20" t="n">
-        <v>12.21</v>
-      </c>
-      <c r="L20" t="n">
-        <v>15.54</v>
-      </c>
-      <c r="M20" t="n">
-        <v>19.37</v>
-      </c>
-      <c r="N20" t="n">
-        <v>8.08</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="1" t="n">
-        <v>19</v>
-      </c>
-      <c r="B21" t="n">
-        <v>24</v>
-      </c>
-      <c r="C21" t="n">
-        <v>0.0068029</v>
-      </c>
-      <c r="D21" t="n">
-        <v>0.35</v>
-      </c>
-      <c r="E21" t="n">
-        <v>2.89</v>
-      </c>
-      <c r="F21" t="n">
-        <v>5.43</v>
-      </c>
-      <c r="G21" t="n">
-        <v>1.22</v>
-      </c>
-      <c r="H21" t="n">
-        <v>3.57</v>
-      </c>
-      <c r="I21" t="n">
-        <v>9.039999999999999</v>
-      </c>
-      <c r="J21" t="n">
-        <v>9.130000000000001</v>
-      </c>
-      <c r="K21" t="n">
-        <v>10.4</v>
-      </c>
-      <c r="L21" t="n">
-        <v>13.27</v>
-      </c>
-      <c r="M21" t="n">
-        <v>16.58</v>
-      </c>
-      <c r="N21" t="n">
-        <v>7.19</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="1" t="n">
-        <v>20</v>
-      </c>
-      <c r="B22" t="n">
-        <v>25</v>
-      </c>
-      <c r="C22" t="n">
-        <v>0.0073346</v>
-      </c>
-      <c r="D22" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="E22" t="n">
-        <v>2.79</v>
-      </c>
-      <c r="F22" t="n">
-        <v>5.24</v>
-      </c>
-      <c r="G22" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="H22" t="n">
-        <v>3.95</v>
-      </c>
-      <c r="I22" t="n">
-        <v>9.529999999999999</v>
-      </c>
-      <c r="J22" t="n">
-        <v>9.77</v>
-      </c>
-      <c r="K22" t="n">
-        <v>11.22</v>
-      </c>
-      <c r="L22" t="n">
-        <v>14.28</v>
-      </c>
-      <c r="M22" t="n">
-        <v>17.8</v>
-      </c>
-      <c r="N22" t="n">
-        <v>7.58</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="1" t="n">
-        <v>21</v>
-      </c>
-      <c r="B23" t="n">
-        <v>26</v>
-      </c>
-      <c r="C23" t="n">
-        <v>0.008988599999999999</v>
-      </c>
-      <c r="D23" t="n">
-        <v>0.43</v>
-      </c>
-      <c r="E23" t="n">
-        <v>3.08</v>
-      </c>
-      <c r="F23" t="n">
-        <v>5.75</v>
-      </c>
-      <c r="G23" t="n">
-        <v>1.66</v>
-      </c>
-      <c r="H23" t="n">
-        <v>3.02</v>
-      </c>
-      <c r="I23" t="n">
-        <v>8.369999999999999</v>
-      </c>
-      <c r="J23" t="n">
-        <v>8.289999999999999</v>
-      </c>
-      <c r="K23" t="n">
-        <v>9.4</v>
-      </c>
-      <c r="L23" t="n">
-        <v>12.09</v>
-      </c>
-      <c r="M23" t="n">
-        <v>15.22</v>
-      </c>
-      <c r="N23" t="n">
-        <v>6.73</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="1" t="n">
-        <v>22</v>
-      </c>
-      <c r="B24" t="n">
-        <v>27</v>
-      </c>
-      <c r="C24" t="n">
-        <v>0.010944</v>
-      </c>
-      <c r="D24" t="n">
-        <v>0.34</v>
-      </c>
-      <c r="E24" t="n">
-        <v>2.86</v>
-      </c>
-      <c r="F24" t="n">
-        <v>5.38</v>
-      </c>
-      <c r="G24" t="n">
-        <v>1.14</v>
-      </c>
-      <c r="H24" t="n">
-        <v>3.7</v>
-      </c>
-      <c r="I24" t="n">
-        <v>9.220000000000001</v>
-      </c>
-      <c r="J24" t="n">
-        <v>9.380000000000001</v>
-      </c>
-      <c r="K24" t="n">
-        <v>10.74</v>
-      </c>
-      <c r="L24" t="n">
-        <v>13.7</v>
-      </c>
-      <c r="M24" t="n">
-        <v>17.13</v>
-      </c>
-      <c r="N24" t="n">
-        <v>7.36</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="1" t="n">
-        <v>23</v>
-      </c>
-      <c r="B25" t="n">
-        <v>28</v>
-      </c>
-      <c r="C25" t="n">
-        <v>0.0067129</v>
-      </c>
-      <c r="D25" t="n">
-        <v>0.29</v>
-      </c>
-      <c r="E25" t="n">
-        <v>2.73</v>
-      </c>
-      <c r="F25" t="n">
-        <v>5.11</v>
-      </c>
-      <c r="G25" t="n">
-        <v>0.71</v>
-      </c>
-      <c r="H25" t="n">
-        <v>4.34</v>
-      </c>
-      <c r="I25" t="n">
-        <v>10.09</v>
-      </c>
-      <c r="J25" t="n">
-        <v>10.58</v>
-      </c>
-      <c r="K25" t="n">
-        <v>12.34</v>
-      </c>
-      <c r="L25" t="n">
-        <v>15.75</v>
-      </c>
-      <c r="M25" t="n">
-        <v>19.68</v>
-      </c>
-      <c r="N25" t="n">
-        <v>8.16</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="1" t="n">
-        <v>24</v>
-      </c>
-      <c r="B26" t="n">
-        <v>29</v>
-      </c>
-      <c r="C26" t="n">
-        <v>0.0070059</v>
-      </c>
-      <c r="D26" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="E26" t="n">
-        <v>2.64</v>
-      </c>
-      <c r="F26" t="n">
-        <v>4.95</v>
-      </c>
-      <c r="G26" t="n">
-        <v>0.48</v>
-      </c>
-      <c r="H26" t="n">
-        <v>4.64</v>
-      </c>
-      <c r="I26" t="n">
-        <v>10.47</v>
-      </c>
-      <c r="J26" t="n">
-        <v>11.09</v>
-      </c>
-      <c r="K26" t="n">
-        <v>12.98</v>
-      </c>
-      <c r="L26" t="n">
-        <v>16.52</v>
-      </c>
-      <c r="M26" t="n">
-        <v>20.61</v>
-      </c>
-      <c r="N26" t="n">
-        <v>8.460000000000001</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="1" t="n">
-        <v>25</v>
-      </c>
-      <c r="B27" t="n">
-        <v>30</v>
-      </c>
-      <c r="C27" t="n">
-        <v>0.0077365</v>
-      </c>
-      <c r="D27" t="n">
-        <v>0.23</v>
-      </c>
-      <c r="E27" t="n">
-        <v>2.59</v>
-      </c>
-      <c r="F27" t="n">
-        <v>4.86</v>
-      </c>
-      <c r="G27" t="n">
-        <v>0.34</v>
-      </c>
-      <c r="H27" t="n">
-        <v>4.84</v>
-      </c>
-      <c r="I27" t="n">
-        <v>10.73</v>
-      </c>
-      <c r="J27" t="n">
-        <v>11.44</v>
-      </c>
-      <c r="K27" t="n">
-        <v>13.44</v>
-      </c>
-      <c r="L27" t="n">
-        <v>17.1</v>
-      </c>
-      <c r="M27" t="n">
-        <v>21.32</v>
-      </c>
-      <c r="N27" t="n">
-        <v>8.69</v>
+        <v>5.66</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated on 11-01-2023 at 18:16
</commit_message>
<xml_diff>
--- a/output/accuracy_cubic.xlsx
+++ b/output/accuracy_cubic.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N17"/>
+  <dimension ref="A1:N27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -474,43 +474,43 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>45</v>
+        <v>5</v>
       </c>
       <c r="C2" t="n">
-        <v>0.032975</v>
+        <v>0.0026477</v>
       </c>
       <c r="D2" t="n">
-        <v>4.31</v>
+        <v>25.33</v>
       </c>
       <c r="E2" t="n">
-        <v>0.26</v>
+        <v>71.02</v>
       </c>
       <c r="F2" t="n">
-        <v>1.91</v>
+        <v>142.76</v>
       </c>
       <c r="G2" t="n">
-        <v>2.73</v>
+        <v>246.23</v>
       </c>
       <c r="H2" t="n">
-        <v>1.42</v>
+        <v>387.13</v>
       </c>
       <c r="I2" t="n">
-        <v>0.55</v>
+        <v>571.13</v>
       </c>
       <c r="J2" t="n">
-        <v>2.95</v>
+        <v>837.27</v>
       </c>
       <c r="K2" t="n">
-        <v>2.4</v>
+        <v>1135.16</v>
       </c>
       <c r="L2" t="n">
-        <v>3.03</v>
+        <v>1495.45</v>
       </c>
       <c r="M2" t="n">
-        <v>0.02</v>
+        <v>1924.03</v>
       </c>
       <c r="N2" t="n">
-        <v>1.96</v>
+        <v>683.55</v>
       </c>
     </row>
     <row r="3">
@@ -518,43 +518,43 @@
         <v>1</v>
       </c>
       <c r="B3" t="n">
-        <v>46</v>
+        <v>6</v>
       </c>
       <c r="C3" t="n">
-        <v>0.038934</v>
+        <v>0.0075386</v>
       </c>
       <c r="D3" t="n">
-        <v>4.34</v>
+        <v>20.13</v>
       </c>
       <c r="E3" t="n">
-        <v>0.37</v>
+        <v>53.82</v>
       </c>
       <c r="F3" t="n">
-        <v>1.65</v>
+        <v>104.33</v>
       </c>
       <c r="G3" t="n">
-        <v>2.26</v>
+        <v>174.94</v>
       </c>
       <c r="H3" t="n">
-        <v>2.14</v>
+        <v>268.92</v>
       </c>
       <c r="I3" t="n">
-        <v>0.51</v>
+        <v>389.54</v>
       </c>
       <c r="J3" t="n">
-        <v>1.45</v>
+        <v>563.66</v>
       </c>
       <c r="K3" t="n">
-        <v>0.43</v>
+        <v>754.13</v>
       </c>
       <c r="L3" t="n">
-        <v>5.43</v>
+        <v>982.38</v>
       </c>
       <c r="M3" t="n">
-        <v>3.12</v>
+        <v>1251.82</v>
       </c>
       <c r="N3" t="n">
-        <v>2.17</v>
+        <v>456.37</v>
       </c>
     </row>
     <row r="4">
@@ -562,43 +562,43 @@
         <v>2</v>
       </c>
       <c r="B4" t="n">
-        <v>47</v>
+        <v>7</v>
       </c>
       <c r="C4" t="n">
-        <v>0.04607</v>
+        <v>0</v>
       </c>
       <c r="D4" t="n">
-        <v>4.35</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="E4" t="n">
-        <v>0.41</v>
+        <v>2.63</v>
       </c>
       <c r="F4" t="n">
-        <v>1.58</v>
+        <v>7.34</v>
       </c>
       <c r="G4" t="n">
-        <v>2.14</v>
+        <v>15.81</v>
       </c>
       <c r="H4" t="n">
-        <v>2.32</v>
+        <v>29.17</v>
       </c>
       <c r="I4" t="n">
-        <v>0.76</v>
+        <v>48.55</v>
       </c>
       <c r="J4" t="n">
-        <v>1.11</v>
+        <v>81.54000000000001</v>
       </c>
       <c r="K4" t="n">
-        <v>0</v>
+        <v>117.64</v>
       </c>
       <c r="L4" t="n">
-        <v>5.94</v>
+        <v>163.49</v>
       </c>
       <c r="M4" t="n">
-        <v>3.76</v>
+        <v>220.27</v>
       </c>
       <c r="N4" t="n">
-        <v>2.24</v>
+        <v>68.7</v>
       </c>
     </row>
     <row r="5">
@@ -606,43 +606,43 @@
         <v>3</v>
       </c>
       <c r="B5" t="n">
-        <v>48</v>
+        <v>8</v>
       </c>
       <c r="C5" t="n">
-        <v>0.054777</v>
+        <v>0.0022368</v>
       </c>
       <c r="D5" t="n">
-        <v>4.36</v>
+        <v>10.98</v>
       </c>
       <c r="E5" t="n">
-        <v>0.41</v>
+        <v>26.91</v>
       </c>
       <c r="F5" t="n">
-        <v>1.58</v>
+        <v>48.69</v>
       </c>
       <c r="G5" t="n">
-        <v>2.15</v>
+        <v>77.18000000000001</v>
       </c>
       <c r="H5" t="n">
-        <v>2.29</v>
+        <v>113.26</v>
       </c>
       <c r="I5" t="n">
-        <v>0.72</v>
+        <v>157.82</v>
       </c>
       <c r="J5" t="n">
-        <v>1.17</v>
+        <v>223.22</v>
       </c>
       <c r="K5" t="n">
-        <v>0.09</v>
+        <v>289.71</v>
       </c>
       <c r="L5" t="n">
-        <v>5.83</v>
+        <v>367.71</v>
       </c>
       <c r="M5" t="n">
-        <v>3.62</v>
+        <v>458.14</v>
       </c>
       <c r="N5" t="n">
-        <v>2.22</v>
+        <v>177.36</v>
       </c>
     </row>
     <row r="6">
@@ -650,43 +650,43 @@
         <v>4</v>
       </c>
       <c r="B6" t="n">
-        <v>49</v>
+        <v>9</v>
       </c>
       <c r="C6" t="n">
-        <v>0.008087199999999999</v>
+        <v>0.011528</v>
       </c>
       <c r="D6" t="n">
-        <v>4.39</v>
+        <v>13.54</v>
       </c>
       <c r="E6" t="n">
-        <v>0.27</v>
+        <v>34.15</v>
       </c>
       <c r="F6" t="n">
-        <v>2.1</v>
+        <v>63.24</v>
       </c>
       <c r="G6" t="n">
-        <v>3.27</v>
+        <v>102.18</v>
       </c>
       <c r="H6" t="n">
-        <v>0.44</v>
+        <v>152.38</v>
       </c>
       <c r="I6" t="n">
-        <v>2.18</v>
+        <v>215.22</v>
       </c>
       <c r="J6" t="n">
-        <v>5.39</v>
+        <v>306.57</v>
       </c>
       <c r="K6" t="n">
-        <v>5.77</v>
+        <v>402.28</v>
       </c>
       <c r="L6" t="n">
-        <v>1.19</v>
+        <v>515.4400000000001</v>
       </c>
       <c r="M6" t="n">
-        <v>5.56</v>
+        <v>647.49</v>
       </c>
       <c r="N6" t="n">
-        <v>3.06</v>
+        <v>245.25</v>
       </c>
     </row>
     <row r="7">
@@ -694,43 +694,43 @@
         <v>5</v>
       </c>
       <c r="B7" t="n">
-        <v>50</v>
+        <v>10</v>
       </c>
       <c r="C7" t="n">
-        <v>0.0081095</v>
+        <v>0.024088</v>
       </c>
       <c r="D7" t="n">
-        <v>4.36</v>
+        <v>12.8</v>
       </c>
       <c r="E7" t="n">
-        <v>0.22</v>
+        <v>31.66</v>
       </c>
       <c r="F7" t="n">
-        <v>2.19</v>
+        <v>57.66</v>
       </c>
       <c r="G7" t="n">
-        <v>3.39</v>
+        <v>91.90000000000001</v>
       </c>
       <c r="H7" t="n">
-        <v>0.29</v>
+        <v>135.47</v>
       </c>
       <c r="I7" t="n">
-        <v>2.36</v>
+        <v>189.45</v>
       </c>
       <c r="J7" t="n">
-        <v>5.62</v>
+        <v>268.01</v>
       </c>
       <c r="K7" t="n">
-        <v>6.04</v>
+        <v>348.95</v>
       </c>
       <c r="L7" t="n">
-        <v>1.49</v>
+        <v>444.07</v>
       </c>
       <c r="M7" t="n">
-        <v>5.92</v>
+        <v>554.49</v>
       </c>
       <c r="N7" t="n">
-        <v>3.19</v>
+        <v>213.45</v>
       </c>
     </row>
     <row r="8">
@@ -738,43 +738,43 @@
         <v>6</v>
       </c>
       <c r="B8" t="n">
-        <v>51</v>
+        <v>11</v>
       </c>
       <c r="C8" t="n">
-        <v>0.0081481</v>
+        <v>0.07047200000000001</v>
       </c>
       <c r="D8" t="n">
-        <v>4.39</v>
+        <v>9.81</v>
       </c>
       <c r="E8" t="n">
-        <v>0.29</v>
+        <v>23.67</v>
       </c>
       <c r="F8" t="n">
-        <v>2.08</v>
+        <v>42.23</v>
       </c>
       <c r="G8" t="n">
-        <v>3.24</v>
+        <v>66.19</v>
       </c>
       <c r="H8" t="n">
-        <v>0.48</v>
+        <v>96.2</v>
       </c>
       <c r="I8" t="n">
-        <v>2.13</v>
+        <v>132.95</v>
       </c>
       <c r="J8" t="n">
-        <v>5.33</v>
+        <v>187.32</v>
       </c>
       <c r="K8" t="n">
-        <v>5.7</v>
+        <v>241.49</v>
       </c>
       <c r="L8" t="n">
-        <v>1.11</v>
+        <v>304.73</v>
       </c>
       <c r="M8" t="n">
-        <v>5.46</v>
+        <v>377.74</v>
       </c>
       <c r="N8" t="n">
-        <v>3.02</v>
+        <v>148.23</v>
       </c>
     </row>
     <row r="9">
@@ -782,43 +782,43 @@
         <v>7</v>
       </c>
       <c r="B9" t="n">
-        <v>52</v>
+        <v>12</v>
       </c>
       <c r="C9" t="n">
-        <v>0.008276499999999999</v>
+        <v>0.11871</v>
       </c>
       <c r="D9" t="n">
-        <v>4.45</v>
+        <v>5.45</v>
       </c>
       <c r="E9" t="n">
-        <v>0.41</v>
+        <v>12.3</v>
       </c>
       <c r="F9" t="n">
-        <v>1.89</v>
+        <v>20.73</v>
       </c>
       <c r="G9" t="n">
-        <v>2.97</v>
+        <v>30.94</v>
       </c>
       <c r="H9" t="n">
-        <v>0.8100000000000001</v>
+        <v>43.14</v>
       </c>
       <c r="I9" t="n">
-        <v>1.7</v>
+        <v>57.5</v>
       </c>
       <c r="J9" t="n">
-        <v>4.81</v>
+        <v>80.65000000000001</v>
       </c>
       <c r="K9" t="n">
-        <v>5.08</v>
+        <v>100.65</v>
       </c>
       <c r="L9" t="n">
-        <v>0.43</v>
+        <v>123.51</v>
       </c>
       <c r="M9" t="n">
-        <v>4.65</v>
+        <v>149.43</v>
       </c>
       <c r="N9" t="n">
-        <v>2.72</v>
+        <v>62.43</v>
       </c>
     </row>
     <row r="10">
@@ -826,43 +826,43 @@
         <v>8</v>
       </c>
       <c r="B10" t="n">
-        <v>53</v>
+        <v>13</v>
       </c>
       <c r="C10" t="n">
-        <v>0.008313900000000001</v>
+        <v>0.13389</v>
       </c>
       <c r="D10" t="n">
-        <v>4.42</v>
+        <v>4.41</v>
       </c>
       <c r="E10" t="n">
-        <v>0.34</v>
+        <v>9.6</v>
       </c>
       <c r="F10" t="n">
-        <v>2</v>
+        <v>15.65</v>
       </c>
       <c r="G10" t="n">
-        <v>3.12</v>
+        <v>22.64</v>
       </c>
       <c r="H10" t="n">
-        <v>0.63</v>
+        <v>30.67</v>
       </c>
       <c r="I10" t="n">
-        <v>1.93</v>
+        <v>39.81</v>
       </c>
       <c r="J10" t="n">
-        <v>5.09</v>
+        <v>55.69</v>
       </c>
       <c r="K10" t="n">
-        <v>5.41</v>
+        <v>67.75</v>
       </c>
       <c r="L10" t="n">
-        <v>0.79</v>
+        <v>81.23</v>
       </c>
       <c r="M10" t="n">
-        <v>5.08</v>
+        <v>96.22</v>
       </c>
       <c r="N10" t="n">
-        <v>2.88</v>
+        <v>42.37</v>
       </c>
     </row>
     <row r="11">
@@ -870,43 +870,43 @@
         <v>9</v>
       </c>
       <c r="B11" t="n">
-        <v>54</v>
+        <v>14</v>
       </c>
       <c r="C11" t="n">
-        <v>0.008314999999999999</v>
+        <v>0.097464</v>
       </c>
       <c r="D11" t="n">
-        <v>4.42</v>
+        <v>2.65</v>
       </c>
       <c r="E11" t="n">
-        <v>0.35</v>
+        <v>5.29</v>
       </c>
       <c r="F11" t="n">
-        <v>1.98</v>
+        <v>7.88</v>
       </c>
       <c r="G11" t="n">
-        <v>3.09</v>
+        <v>10.4</v>
       </c>
       <c r="H11" t="n">
-        <v>0.66</v>
+        <v>12.81</v>
       </c>
       <c r="I11" t="n">
-        <v>1.89</v>
+        <v>15.09</v>
       </c>
       <c r="J11" t="n">
-        <v>5.04</v>
+        <v>21.53</v>
       </c>
       <c r="K11" t="n">
-        <v>5.35</v>
+        <v>23.52</v>
       </c>
       <c r="L11" t="n">
-        <v>0.73</v>
+        <v>25.28</v>
       </c>
       <c r="M11" t="n">
-        <v>5.01</v>
+        <v>26.78</v>
       </c>
       <c r="N11" t="n">
-        <v>2.85</v>
+        <v>15.12</v>
       </c>
     </row>
     <row r="12">
@@ -914,43 +914,43 @@
         <v>10</v>
       </c>
       <c r="B12" t="n">
-        <v>55</v>
+        <v>15</v>
       </c>
       <c r="C12" t="n">
-        <v>0.0083599</v>
+        <v>0.09748900000000001</v>
       </c>
       <c r="D12" t="n">
-        <v>4.39</v>
+        <v>2.62</v>
       </c>
       <c r="E12" t="n">
-        <v>0.28</v>
+        <v>5.21</v>
       </c>
       <c r="F12" t="n">
-        <v>2.09</v>
+        <v>7.74</v>
       </c>
       <c r="G12" t="n">
-        <v>3.25</v>
+        <v>10.17</v>
       </c>
       <c r="H12" t="n">
-        <v>0.47</v>
+        <v>12.47</v>
       </c>
       <c r="I12" t="n">
-        <v>2.14</v>
+        <v>14.61</v>
       </c>
       <c r="J12" t="n">
-        <v>5.34</v>
+        <v>20.86</v>
       </c>
       <c r="K12" t="n">
-        <v>5.71</v>
+        <v>22.65</v>
       </c>
       <c r="L12" t="n">
-        <v>1.12</v>
+        <v>24.17</v>
       </c>
       <c r="M12" t="n">
-        <v>5.48</v>
+        <v>25.4</v>
       </c>
       <c r="N12" t="n">
-        <v>3.03</v>
+        <v>14.59</v>
       </c>
     </row>
     <row r="13">
@@ -958,43 +958,43 @@
         <v>11</v>
       </c>
       <c r="B13" t="n">
-        <v>56</v>
+        <v>16</v>
       </c>
       <c r="C13" t="n">
-        <v>0.0075223</v>
+        <v>0.14202</v>
       </c>
       <c r="D13" t="n">
-        <v>4.25</v>
+        <v>3.62</v>
       </c>
       <c r="E13" t="n">
-        <v>0.02</v>
+        <v>7.58</v>
       </c>
       <c r="F13" t="n">
-        <v>2.57</v>
+        <v>11.9</v>
       </c>
       <c r="G13" t="n">
-        <v>3.92</v>
+        <v>16.6</v>
       </c>
       <c r="H13" t="n">
-        <v>0.36</v>
+        <v>21.68</v>
       </c>
       <c r="I13" t="n">
-        <v>3.18</v>
+        <v>27.17</v>
       </c>
       <c r="J13" t="n">
-        <v>6.62</v>
+        <v>37.99</v>
       </c>
       <c r="K13" t="n">
-        <v>7.21</v>
+        <v>44.56</v>
       </c>
       <c r="L13" t="n">
-        <v>2.76</v>
+        <v>51.6</v>
       </c>
       <c r="M13" t="n">
-        <v>7.41</v>
+        <v>59.12</v>
       </c>
       <c r="N13" t="n">
-        <v>3.83</v>
+        <v>28.18</v>
       </c>
     </row>
     <row r="14">
@@ -1002,43 +1002,43 @@
         <v>12</v>
       </c>
       <c r="B14" t="n">
-        <v>57</v>
+        <v>17</v>
       </c>
       <c r="C14" t="n">
-        <v>0.0075373</v>
+        <v>0.33976</v>
       </c>
       <c r="D14" t="n">
-        <v>4.23</v>
+        <v>0.98</v>
       </c>
       <c r="E14" t="n">
-        <v>0.07000000000000001</v>
+        <v>1.25</v>
       </c>
       <c r="F14" t="n">
-        <v>2.64</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="G14" t="n">
-        <v>4.01</v>
+        <v>0.83</v>
       </c>
       <c r="H14" t="n">
-        <v>0.47</v>
+        <v>3.42</v>
       </c>
       <c r="I14" t="n">
-        <v>3.32</v>
+        <v>7.21</v>
       </c>
       <c r="J14" t="n">
-        <v>6.8</v>
+        <v>9.08</v>
       </c>
       <c r="K14" t="n">
-        <v>7.41</v>
+        <v>15.88</v>
       </c>
       <c r="L14" t="n">
-        <v>2.99</v>
+        <v>24.29</v>
       </c>
       <c r="M14" t="n">
-        <v>7.68</v>
+        <v>34.44</v>
       </c>
       <c r="N14" t="n">
-        <v>3.96</v>
+        <v>9.81</v>
       </c>
     </row>
     <row r="15">
@@ -1046,43 +1046,43 @@
         <v>13</v>
       </c>
       <c r="B15" t="n">
-        <v>58</v>
+        <v>18</v>
       </c>
       <c r="C15" t="n">
-        <v>0.0078018</v>
+        <v>0.26889</v>
       </c>
       <c r="D15" t="n">
-        <v>4.15</v>
+        <v>3.97</v>
       </c>
       <c r="E15" t="n">
-        <v>0.23</v>
+        <v>8.65</v>
       </c>
       <c r="F15" t="n">
-        <v>2.9</v>
+        <v>14.12</v>
       </c>
       <c r="G15" t="n">
-        <v>4.38</v>
+        <v>20.47</v>
       </c>
       <c r="H15" t="n">
-        <v>0.93</v>
+        <v>27.79</v>
       </c>
       <c r="I15" t="n">
-        <v>3.89</v>
+        <v>36.15</v>
       </c>
       <c r="J15" t="n">
-        <v>7.51</v>
+        <v>51.02</v>
       </c>
       <c r="K15" t="n">
-        <v>8.25</v>
+        <v>62.14</v>
       </c>
       <c r="L15" t="n">
-        <v>3.91</v>
+        <v>74.59999999999999</v>
       </c>
       <c r="M15" t="n">
-        <v>8.77</v>
+        <v>88.48999999999999</v>
       </c>
       <c r="N15" t="n">
-        <v>4.49</v>
+        <v>38.74</v>
       </c>
     </row>
     <row r="16">
@@ -1090,43 +1090,43 @@
         <v>14</v>
       </c>
       <c r="B16" t="n">
-        <v>59</v>
+        <v>19</v>
       </c>
       <c r="C16" t="n">
-        <v>0.008195300000000001</v>
+        <v>0.27845</v>
       </c>
       <c r="D16" t="n">
-        <v>4.06</v>
+        <v>4.77</v>
       </c>
       <c r="E16" t="n">
-        <v>0.43</v>
+        <v>10.45</v>
       </c>
       <c r="F16" t="n">
-        <v>3.22</v>
+        <v>17.15</v>
       </c>
       <c r="G16" t="n">
-        <v>4.82</v>
+        <v>24.97</v>
       </c>
       <c r="H16" t="n">
-        <v>1.47</v>
+        <v>34.01</v>
       </c>
       <c r="I16" t="n">
-        <v>4.58</v>
+        <v>44.36</v>
       </c>
       <c r="J16" t="n">
-        <v>8.359999999999999</v>
+        <v>61.88</v>
       </c>
       <c r="K16" t="n">
-        <v>9.24</v>
+        <v>75.65000000000001</v>
       </c>
       <c r="L16" t="n">
-        <v>5</v>
+        <v>91.09999999999999</v>
       </c>
       <c r="M16" t="n">
-        <v>10.07</v>
+        <v>108.32</v>
       </c>
       <c r="N16" t="n">
-        <v>5.12</v>
+        <v>47.27</v>
       </c>
     </row>
     <row r="17">
@@ -1134,43 +1134,483 @@
         <v>15</v>
       </c>
       <c r="B17" t="n">
-        <v>60</v>
+        <v>20</v>
       </c>
       <c r="C17" t="n">
-        <v>0.0084901</v>
+        <v>0.31894</v>
       </c>
       <c r="D17" t="n">
-        <v>3.98</v>
+        <v>4.76</v>
       </c>
       <c r="E17" t="n">
-        <v>0.6</v>
+        <v>10.39</v>
       </c>
       <c r="F17" t="n">
-        <v>3.49</v>
+        <v>16.98</v>
       </c>
       <c r="G17" t="n">
-        <v>5.18</v>
+        <v>24.61</v>
       </c>
       <c r="H17" t="n">
-        <v>1.93</v>
+        <v>33.38</v>
       </c>
       <c r="I17" t="n">
-        <v>5.16</v>
+        <v>43.37</v>
       </c>
       <c r="J17" t="n">
-        <v>9.07</v>
+        <v>60.38</v>
       </c>
       <c r="K17" t="n">
-        <v>10.08</v>
+        <v>73.56</v>
       </c>
       <c r="L17" t="n">
-        <v>5.92</v>
+        <v>88.29000000000001</v>
       </c>
       <c r="M17" t="n">
-        <v>11.15</v>
+        <v>104.66</v>
       </c>
       <c r="N17" t="n">
-        <v>5.66</v>
+        <v>46.04</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="1" t="n">
+        <v>16</v>
+      </c>
+      <c r="B18" t="n">
+        <v>21</v>
+      </c>
+      <c r="C18" t="n">
+        <v>0.34913</v>
+      </c>
+      <c r="D18" t="n">
+        <v>2.12</v>
+      </c>
+      <c r="E18" t="n">
+        <v>4.16</v>
+      </c>
+      <c r="F18" t="n">
+        <v>6.12</v>
+      </c>
+      <c r="G18" t="n">
+        <v>7.97</v>
+      </c>
+      <c r="H18" t="n">
+        <v>9.73</v>
+      </c>
+      <c r="I18" t="n">
+        <v>11.37</v>
+      </c>
+      <c r="J18" t="n">
+        <v>17.04</v>
+      </c>
+      <c r="K18" t="n">
+        <v>18.47</v>
+      </c>
+      <c r="L18" t="n">
+        <v>19.75</v>
+      </c>
+      <c r="M18" t="n">
+        <v>20.87</v>
+      </c>
+      <c r="N18" t="n">
+        <v>11.76</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="1" t="n">
+        <v>17</v>
+      </c>
+      <c r="B19" t="n">
+        <v>22</v>
+      </c>
+      <c r="C19" t="n">
+        <v>0.36302</v>
+      </c>
+      <c r="D19" t="n">
+        <v>1.82</v>
+      </c>
+      <c r="E19" t="n">
+        <v>3.46</v>
+      </c>
+      <c r="F19" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="G19" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="H19" t="n">
+        <v>7.06</v>
+      </c>
+      <c r="I19" t="n">
+        <v>7.75</v>
+      </c>
+      <c r="J19" t="n">
+        <v>12.14</v>
+      </c>
+      <c r="K19" t="n">
+        <v>12.23</v>
+      </c>
+      <c r="L19" t="n">
+        <v>11.97</v>
+      </c>
+      <c r="M19" t="n">
+        <v>11.35</v>
+      </c>
+      <c r="N19" t="n">
+        <v>7.88</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="1" t="n">
+        <v>18</v>
+      </c>
+      <c r="B20" t="n">
+        <v>23</v>
+      </c>
+      <c r="C20" t="n">
+        <v>0.46354</v>
+      </c>
+      <c r="D20" t="n">
+        <v>2.08</v>
+      </c>
+      <c r="E20" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="F20" t="n">
+        <v>6.03</v>
+      </c>
+      <c r="G20" t="n">
+        <v>7.87</v>
+      </c>
+      <c r="H20" t="n">
+        <v>9.6</v>
+      </c>
+      <c r="I20" t="n">
+        <v>11.23</v>
+      </c>
+      <c r="J20" t="n">
+        <v>16.9</v>
+      </c>
+      <c r="K20" t="n">
+        <v>18.33</v>
+      </c>
+      <c r="L20" t="n">
+        <v>19.62</v>
+      </c>
+      <c r="M20" t="n">
+        <v>20.75</v>
+      </c>
+      <c r="N20" t="n">
+        <v>11.65</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="1" t="n">
+        <v>19</v>
+      </c>
+      <c r="B21" t="n">
+        <v>24</v>
+      </c>
+      <c r="C21" t="n">
+        <v>0.43849</v>
+      </c>
+      <c r="D21" t="n">
+        <v>3</v>
+      </c>
+      <c r="E21" t="n">
+        <v>6.32</v>
+      </c>
+      <c r="F21" t="n">
+        <v>9.970000000000001</v>
+      </c>
+      <c r="G21" t="n">
+        <v>14</v>
+      </c>
+      <c r="H21" t="n">
+        <v>18.44</v>
+      </c>
+      <c r="I21" t="n">
+        <v>23.32</v>
+      </c>
+      <c r="J21" t="n">
+        <v>33.42</v>
+      </c>
+      <c r="K21" t="n">
+        <v>39.5</v>
+      </c>
+      <c r="L21" t="n">
+        <v>46.14</v>
+      </c>
+      <c r="M21" t="n">
+        <v>53.38</v>
+      </c>
+      <c r="N21" t="n">
+        <v>24.75</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="1" t="n">
+        <v>20</v>
+      </c>
+      <c r="B22" t="n">
+        <v>25</v>
+      </c>
+      <c r="C22" t="n">
+        <v>0.45643</v>
+      </c>
+      <c r="D22" t="n">
+        <v>3.43</v>
+      </c>
+      <c r="E22" t="n">
+        <v>7.27</v>
+      </c>
+      <c r="F22" t="n">
+        <v>11.56</v>
+      </c>
+      <c r="G22" t="n">
+        <v>16.33</v>
+      </c>
+      <c r="H22" t="n">
+        <v>21.64</v>
+      </c>
+      <c r="I22" t="n">
+        <v>27.51</v>
+      </c>
+      <c r="J22" t="n">
+        <v>38.93</v>
+      </c>
+      <c r="K22" t="n">
+        <v>46.31</v>
+      </c>
+      <c r="L22" t="n">
+        <v>54.41</v>
+      </c>
+      <c r="M22" t="n">
+        <v>63.26</v>
+      </c>
+      <c r="N22" t="n">
+        <v>29.06</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="1" t="n">
+        <v>21</v>
+      </c>
+      <c r="B23" t="n">
+        <v>26</v>
+      </c>
+      <c r="C23" t="n">
+        <v>0.5197000000000001</v>
+      </c>
+      <c r="D23" t="n">
+        <v>2.91</v>
+      </c>
+      <c r="E23" t="n">
+        <v>6.06</v>
+      </c>
+      <c r="F23" t="n">
+        <v>9.470000000000001</v>
+      </c>
+      <c r="G23" t="n">
+        <v>13.16</v>
+      </c>
+      <c r="H23" t="n">
+        <v>17.14</v>
+      </c>
+      <c r="I23" t="n">
+        <v>21.45</v>
+      </c>
+      <c r="J23" t="n">
+        <v>30.76</v>
+      </c>
+      <c r="K23" t="n">
+        <v>35.97</v>
+      </c>
+      <c r="L23" t="n">
+        <v>41.59</v>
+      </c>
+      <c r="M23" t="n">
+        <v>47.63</v>
+      </c>
+      <c r="N23" t="n">
+        <v>22.62</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="1" t="n">
+        <v>22</v>
+      </c>
+      <c r="B24" t="n">
+        <v>27</v>
+      </c>
+      <c r="C24" t="n">
+        <v>0.57867</v>
+      </c>
+      <c r="D24" t="n">
+        <v>2.14</v>
+      </c>
+      <c r="E24" t="n">
+        <v>4.27</v>
+      </c>
+      <c r="F24" t="n">
+        <v>6.39</v>
+      </c>
+      <c r="G24" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="H24" t="n">
+        <v>10.6</v>
+      </c>
+      <c r="I24" t="n">
+        <v>12.7</v>
+      </c>
+      <c r="J24" t="n">
+        <v>19.02</v>
+      </c>
+      <c r="K24" t="n">
+        <v>21.18</v>
+      </c>
+      <c r="L24" t="n">
+        <v>23.34</v>
+      </c>
+      <c r="M24" t="n">
+        <v>25.5</v>
+      </c>
+      <c r="N24" t="n">
+        <v>13.36</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="1" t="n">
+        <v>23</v>
+      </c>
+      <c r="B25" t="n">
+        <v>28</v>
+      </c>
+      <c r="C25" t="n">
+        <v>0.51812</v>
+      </c>
+      <c r="D25" t="n">
+        <v>2</v>
+      </c>
+      <c r="E25" t="n">
+        <v>3.92</v>
+      </c>
+      <c r="F25" t="n">
+        <v>5.76</v>
+      </c>
+      <c r="G25" t="n">
+        <v>7.51</v>
+      </c>
+      <c r="H25" t="n">
+        <v>9.17</v>
+      </c>
+      <c r="I25" t="n">
+        <v>10.73</v>
+      </c>
+      <c r="J25" t="n">
+        <v>16.32</v>
+      </c>
+      <c r="K25" t="n">
+        <v>17.71</v>
+      </c>
+      <c r="L25" t="n">
+        <v>18.98</v>
+      </c>
+      <c r="M25" t="n">
+        <v>20.13</v>
+      </c>
+      <c r="N25" t="n">
+        <v>11.22</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="1" t="n">
+        <v>24</v>
+      </c>
+      <c r="B26" t="n">
+        <v>29</v>
+      </c>
+      <c r="C26" t="n">
+        <v>0.5415</v>
+      </c>
+      <c r="D26" t="n">
+        <v>1.82</v>
+      </c>
+      <c r="E26" t="n">
+        <v>3.51</v>
+      </c>
+      <c r="F26" t="n">
+        <v>5.06</v>
+      </c>
+      <c r="G26" t="n">
+        <v>6.47</v>
+      </c>
+      <c r="H26" t="n">
+        <v>7.72</v>
+      </c>
+      <c r="I26" t="n">
+        <v>8.800000000000001</v>
+      </c>
+      <c r="J26" t="n">
+        <v>13.76</v>
+      </c>
+      <c r="K26" t="n">
+        <v>14.5</v>
+      </c>
+      <c r="L26" t="n">
+        <v>15.05</v>
+      </c>
+      <c r="M26" t="n">
+        <v>15.37</v>
+      </c>
+      <c r="N26" t="n">
+        <v>9.210000000000001</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="1" t="n">
+        <v>25</v>
+      </c>
+      <c r="B27" t="n">
+        <v>30</v>
+      </c>
+      <c r="C27" t="n">
+        <v>0.55535</v>
+      </c>
+      <c r="D27" t="n">
+        <v>1.95</v>
+      </c>
+      <c r="E27" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="F27" t="n">
+        <v>5.56</v>
+      </c>
+      <c r="G27" t="n">
+        <v>7.21</v>
+      </c>
+      <c r="H27" t="n">
+        <v>8.75</v>
+      </c>
+      <c r="I27" t="n">
+        <v>10.16</v>
+      </c>
+      <c r="J27" t="n">
+        <v>15.56</v>
+      </c>
+      <c r="K27" t="n">
+        <v>16.76</v>
+      </c>
+      <c r="L27" t="n">
+        <v>17.81</v>
+      </c>
+      <c r="M27" t="n">
+        <v>18.71</v>
+      </c>
+      <c r="N27" t="n">
+        <v>10.63</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated on 11-05-2023 at 12:12
</commit_message>
<xml_diff>
--- a/output/accuracy_cubic.xlsx
+++ b/output/accuracy_cubic.xlsx
@@ -1,138 +1,163 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4506"/>
+  <fileSharing readOnlyRecommended="0" userName="Gustavo"/>
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView activeTab="0" xWindow="240" yWindow="60" windowWidth="0" windowHeight="0" tabRatio="500"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId3"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr/>
+  <extLst>
+    <ext uri="smNativeData">
+      <pm:revision xmlns:pm="smNativeData" day="1699202731" val="1066" rev="124" revOS="4" revMin="124" revMax="0"/>
+      <pm:docPrefs xmlns:pm="smNativeData" id="1699202731" fixedDigits="0" showNotice="1" showFrameBounds="1" autoChart="1" recalcOnPrint="1" recalcOnCopy="1" finalRounding="1" compatTextArt="1" tab="567" useDefinedPrintRange="1" printArea="currentSheet"/>
+      <pm:compatibility xmlns:pm="smNativeData" id="1699202731" overlapCells="1"/>
+      <pm:defCurrency xmlns:pm="smNativeData" id="1699202731"/>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="2">
+  <numFmts count="8">
+    <numFmt numFmtId="5" formatCode="#,##0\ &quot;$&quot;;\-#,##0\ &quot;$&quot;"/>
+    <numFmt numFmtId="6" formatCode="#,##0\ &quot;$&quot;;[Red]\-#,##0\ &quot;$&quot;"/>
+    <numFmt numFmtId="7" formatCode="#,##0.00\ &quot;$&quot;;\-#,##0.00\ &quot;$&quot;"/>
+    <numFmt numFmtId="8" formatCode="#,##0.00\ &quot;$&quot;;[Red]\-#,##0.00\ &quot;$&quot;"/>
+    <numFmt numFmtId="42" formatCode="_-* #,##0\ &quot;$&quot;_-;\-* #,##0\ &quot;$&quot;_-;_-* &quot;-&quot;\ &quot;$&quot;_-;_-@_-"/>
+    <numFmt numFmtId="41" formatCode="_-* #,##0\ _$_-;\-* #,##0\ _$_-;_-* &quot;-&quot;\ _$_-;_-@_-"/>
+    <numFmt numFmtId="44" formatCode="_-* #,##0.00\ &quot;$&quot;_-;\-* #,##0.00\ &quot;$&quot;_-;_-* &quot;-&quot;??\ &quot;$&quot;_-;_-@_-"/>
+    <numFmt numFmtId="43" formatCode="_-* #,##0.00\ _$_-;\-* #,##0.00\ _$_-;_-* &quot;-&quot;??\ _$_-;_-@_-"/>
+  </numFmts>
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
-      <color theme="1"/>
+      <color rgb="FF000000"/>
       <sz val="11"/>
-      <scheme val="minor"/>
+      <extLst>
+        <ext uri="smNativeData">
+          <pm:charSpec xmlns:pm="smNativeData" id="1699202731" ulstyle="none" kern="1">
+            <pm:latin face="Calibri" sz="220" lang="default"/>
+            <pm:cs face="Times New Roman" sz="220" lang="default"/>
+            <pm:ea face="SimSun" sz="220" lang="default"/>
+          </pm:charSpec>
+        </ext>
+      </extLst>
     </font>
     <font>
-      <b val="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <color rgb="FF000000"/>
+      <sz val="10"/>
+      <extLst>
+        <ext uri="smNativeData">
+          <pm:charSpec xmlns:pm="smNativeData" id="1699202731" ulstyle="none" kern="1">
+            <pm:latin face="Arial" sz="200" lang="default"/>
+            <pm:cs face="Times New Roman" sz="200" lang="default"/>
+            <pm:ea face="SimSun" sz="200" lang="default"/>
+          </pm:charSpec>
+        </ext>
+      </extLst>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <family val="2"/>
+      <b/>
+      <color rgb="FF000000"/>
+      <sz val="10"/>
+      <extLst>
+        <ext uri="smNativeData">
+          <pm:charSpec xmlns:pm="smNativeData" id="1699202731" ulstyle="none" kern="1">
+            <pm:latin face="Arial" sz="200" lang="default" weight="bold"/>
+            <pm:cs face="Times New Roman" sz="200" lang="default" weight="bold"/>
+            <pm:ea face="SimSun" sz="200" lang="default" weight="bold"/>
+          </pm:charSpec>
+        </ext>
+      </extLst>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="none"/>
+    </fill>
   </fills>
   <borders count="2">
     <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
+      <left style="none">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="none">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="none">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="none">
+        <color rgb="FF000000"/>
+      </bottom>
+      <extLst>
+        <ext uri="smNativeData">
+          <pm:border xmlns:pm="smNativeData" id="1699202731"/>
+        </ext>
+      </extLst>
     </border>
     <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <extLst>
+        <ext uri="smNativeData">
+          <pm:border xmlns:pm="smNativeData" id="1699202731">
+            <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
+            <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
+            <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
+            <pm:line position="right" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
+          </pm:border>
+        </ext>
+      </extLst>
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
   </cellStyleXfs>
   <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0" customBuiltin="1"/>
   </cellStyles>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
+  <tableStyles count="0"/>
+  <extLst>
+    <ext uri="smNativeData">
+      <pm:charStyles xmlns:pm="smNativeData" id="1699202731" count="1">
+        <pm:charStyle name="Normal" fontId="0" Id="1"/>
+      </pm:charStyles>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -147,10 +172,10 @@
         <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="1F497D"/>
+        <a:srgbClr val="EEECE1"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="EEECE1"/>
+        <a:srgbClr val="1F497D"/>
       </a:lt2>
       <a:accent1>
         <a:srgbClr val="4F81BD"/>
@@ -182,69 +207,11 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Times New Roman"/>
-        <a:font script="Hebr" typeface="Times New Roman"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="MoolBoran"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Times New Roman"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Arial"/>
-        <a:font script="Hebr" typeface="Arial"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="DaunPenh"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Arial"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:ea typeface="SimSun"/>
+        <a:cs typeface="Times New Roman"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -414,21 +381,46 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults/>
+  <a:objectDefaults>
+    <a:spDef>
+      <a:spPr/>
+      <a:bodyPr>
+        <a:prstTxWarp prst="textNoShape">
+          <a:avLst/>
+        </a:prstTxWarp>
+        <a:noAutofit/>
+      </a:bodyPr>
+      <a:lstStyle>
+        <a:defPPr>
+          <a:defRPr/>
+        </a:defPPr>
+      </a:lstStyle>
+      <a:style>
+        <a:lnRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </a:style>
+    </a:spDef>
+  </a:objectDefaults>
   <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <dimension ref="A1:N27"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15.40"/>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="2:14">
       <c r="B1" s="1" t="n">
         <v>0</v>
       </c>
@@ -469,7 +461,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:14">
       <c r="A2" s="1" t="n">
         <v>0</v>
       </c>
@@ -477,43 +469,43 @@
         <v>5</v>
       </c>
       <c r="C2" t="n">
-        <v>0.0026477</v>
+        <v>0.0026476999999999995</v>
       </c>
       <c r="D2" t="n">
-        <v>25.33</v>
+        <v>25.3299999999999983</v>
       </c>
       <c r="E2" t="n">
-        <v>71.02</v>
+        <v>71.019999999999996</v>
       </c>
       <c r="F2" t="n">
-        <v>142.76</v>
+        <v>142.759999999999991</v>
       </c>
       <c r="G2" t="n">
-        <v>246.23</v>
+        <v>246.22999999999999</v>
       </c>
       <c r="H2" t="n">
-        <v>387.13</v>
+        <v>387.129999999999995</v>
       </c>
       <c r="I2" t="n">
-        <v>571.13</v>
+        <v>571.129999999999995</v>
       </c>
       <c r="J2" t="n">
-        <v>837.27</v>
+        <v>837.269999999999982</v>
       </c>
       <c r="K2" t="n">
-        <v>1135.16</v>
+        <v>1135.16000000000008</v>
       </c>
       <c r="L2" t="n">
-        <v>1495.45</v>
+        <v>1495.45000000000005</v>
       </c>
       <c r="M2" t="n">
-        <v>1924.03</v>
+        <v>1924.02999999999997</v>
       </c>
       <c r="N2" t="n">
-        <v>683.55</v>
-      </c>
-    </row>
-    <row r="3">
+        <v>683.549999999999955</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14">
       <c r="A3" s="1" t="n">
         <v>1</v>
       </c>
@@ -521,43 +513,43 @@
         <v>6</v>
       </c>
       <c r="C3" t="n">
-        <v>0.0075386</v>
+        <v>0.00753860000000000063</v>
       </c>
       <c r="D3" t="n">
-        <v>20.13</v>
+        <v>20.129999999999999</v>
       </c>
       <c r="E3" t="n">
-        <v>53.82</v>
+        <v>53.8200000000000003</v>
       </c>
       <c r="F3" t="n">
-        <v>104.33</v>
+        <v>104.329999999999998</v>
       </c>
       <c r="G3" t="n">
-        <v>174.94</v>
+        <v>174.939999999999998</v>
       </c>
       <c r="H3" t="n">
-        <v>268.92</v>
+        <v>268.920000000000016</v>
       </c>
       <c r="I3" t="n">
-        <v>389.54</v>
+        <v>389.54000000000002</v>
       </c>
       <c r="J3" t="n">
-        <v>563.66</v>
+        <v>563.659999999999968</v>
       </c>
       <c r="K3" t="n">
-        <v>754.13</v>
+        <v>754.129999999999995</v>
       </c>
       <c r="L3" t="n">
-        <v>982.38</v>
+        <v>982.380000000000109</v>
       </c>
       <c r="M3" t="n">
-        <v>1251.82</v>
+        <v>1251.81999999999994</v>
       </c>
       <c r="N3" t="n">
-        <v>456.37</v>
-      </c>
-    </row>
-    <row r="4">
+        <v>456.370000000000005</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14">
       <c r="A4" s="1" t="n">
         <v>2</v>
       </c>
@@ -568,40 +560,40 @@
         <v>0</v>
       </c>
       <c r="D4" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.560000000000000053</v>
       </c>
       <c r="E4" t="n">
-        <v>2.63</v>
+        <v>2.62999999999999989</v>
       </c>
       <c r="F4" t="n">
-        <v>7.34</v>
+        <v>7.33999999999999986</v>
       </c>
       <c r="G4" t="n">
-        <v>15.81</v>
+        <v>15.8100000000000005</v>
       </c>
       <c r="H4" t="n">
-        <v>29.17</v>
+        <v>29.1700000000000017</v>
       </c>
       <c r="I4" t="n">
-        <v>48.55</v>
+        <v>48.5499999999999972</v>
       </c>
       <c r="J4" t="n">
-        <v>81.54000000000001</v>
+        <v>81.5400000000000063</v>
       </c>
       <c r="K4" t="n">
-        <v>117.64</v>
+        <v>117.640000000000001</v>
       </c>
       <c r="L4" t="n">
-        <v>163.49</v>
+        <v>163.490000000000009</v>
       </c>
       <c r="M4" t="n">
-        <v>220.27</v>
+        <v>220.27000000000001</v>
       </c>
       <c r="N4" t="n">
-        <v>68.7</v>
-      </c>
-    </row>
-    <row r="5">
+        <v>68.7000000000000028</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14">
       <c r="A5" s="1" t="n">
         <v>3</v>
       </c>
@@ -609,43 +601,43 @@
         <v>8</v>
       </c>
       <c r="C5" t="n">
-        <v>0.0022368</v>
+        <v>0.00223680000000000012</v>
       </c>
       <c r="D5" t="n">
-        <v>10.98</v>
+        <v>10.9800000000000004</v>
       </c>
       <c r="E5" t="n">
-        <v>26.91</v>
+        <v>26.9100000000000001</v>
       </c>
       <c r="F5" t="n">
-        <v>48.69</v>
+        <v>48.6899999999999977</v>
       </c>
       <c r="G5" t="n">
-        <v>77.18000000000001</v>
+        <v>77.1800000000000068</v>
       </c>
       <c r="H5" t="n">
-        <v>113.26</v>
+        <v>113.260000000000005</v>
       </c>
       <c r="I5" t="n">
-        <v>157.82</v>
+        <v>157.819999999999993</v>
       </c>
       <c r="J5" t="n">
-        <v>223.22</v>
+        <v>223.219999999999999</v>
       </c>
       <c r="K5" t="n">
-        <v>289.71</v>
+        <v>289.70999999999998</v>
       </c>
       <c r="L5" t="n">
-        <v>367.71</v>
+        <v>367.70999999999998</v>
       </c>
       <c r="M5" t="n">
-        <v>458.14</v>
+        <v>458.139999999999986</v>
       </c>
       <c r="N5" t="n">
-        <v>177.36</v>
-      </c>
-    </row>
-    <row r="6">
+        <v>177.360000000000014</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14">
       <c r="A6" s="1" t="n">
         <v>4</v>
       </c>
@@ -653,43 +645,43 @@
         <v>9</v>
       </c>
       <c r="C6" t="n">
-        <v>0.011528</v>
+        <v>0.0115280000000000005</v>
       </c>
       <c r="D6" t="n">
-        <v>13.54</v>
+        <v>13.5399999999999991</v>
       </c>
       <c r="E6" t="n">
-        <v>34.15</v>
+        <v>34.1499999999999986</v>
       </c>
       <c r="F6" t="n">
-        <v>63.24</v>
+        <v>63.240000000000002</v>
       </c>
       <c r="G6" t="n">
-        <v>102.18</v>
+        <v>102.180000000000007</v>
       </c>
       <c r="H6" t="n">
-        <v>152.38</v>
+        <v>152.379999999999995</v>
       </c>
       <c r="I6" t="n">
-        <v>215.22</v>
+        <v>215.219999999999999</v>
       </c>
       <c r="J6" t="n">
-        <v>306.57</v>
+        <v>306.569999999999993</v>
       </c>
       <c r="K6" t="n">
-        <v>402.28</v>
+        <v>402.279999999999973</v>
       </c>
       <c r="L6" t="n">
-        <v>515.4400000000001</v>
+        <v>515.440000000000055</v>
       </c>
       <c r="M6" t="n">
-        <v>647.49</v>
+        <v>647.490000000000009</v>
       </c>
       <c r="N6" t="n">
         <v>245.25</v>
       </c>
     </row>
-    <row r="7">
+    <row r="7" spans="1:14">
       <c r="A7" s="1" t="n">
         <v>5</v>
       </c>
@@ -697,43 +689,43 @@
         <v>10</v>
       </c>
       <c r="C7" t="n">
-        <v>0.024088</v>
+        <v>0.0240879999999999983</v>
       </c>
       <c r="D7" t="n">
-        <v>12.8</v>
+        <v>12.8000000000000007</v>
       </c>
       <c r="E7" t="n">
-        <v>31.66</v>
+        <v>31.6600000000000001</v>
       </c>
       <c r="F7" t="n">
-        <v>57.66</v>
+        <v>57.6599999999999966</v>
       </c>
       <c r="G7" t="n">
-        <v>91.90000000000001</v>
+        <v>91.9000000000000057</v>
       </c>
       <c r="H7" t="n">
-        <v>135.47</v>
+        <v>135.470000000000027</v>
       </c>
       <c r="I7" t="n">
-        <v>189.45</v>
+        <v>189.449999999999989</v>
       </c>
       <c r="J7" t="n">
-        <v>268.01</v>
+        <v>268.009999999999991</v>
       </c>
       <c r="K7" t="n">
-        <v>348.95</v>
+        <v>348.949999999999989</v>
       </c>
       <c r="L7" t="n">
-        <v>444.07</v>
+        <v>444.069999999999993</v>
       </c>
       <c r="M7" t="n">
-        <v>554.49</v>
+        <v>554.490000000000009</v>
       </c>
       <c r="N7" t="n">
-        <v>213.45</v>
-      </c>
-    </row>
-    <row r="8">
+        <v>213.449999999999989</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14">
       <c r="A8" s="1" t="n">
         <v>6</v>
       </c>
@@ -741,43 +733,43 @@
         <v>11</v>
       </c>
       <c r="C8" t="n">
-        <v>0.07047200000000001</v>
+        <v>0.0704720000000000013</v>
       </c>
       <c r="D8" t="n">
-        <v>9.81</v>
+        <v>9.8100000000000005</v>
       </c>
       <c r="E8" t="n">
-        <v>23.67</v>
+        <v>23.6700000000000017</v>
       </c>
       <c r="F8" t="n">
-        <v>42.23</v>
+        <v>42.2299999999999969</v>
       </c>
       <c r="G8" t="n">
-        <v>66.19</v>
+        <v>66.1899999999999977</v>
       </c>
       <c r="H8" t="n">
-        <v>96.2</v>
+        <v>96.2000000000000028</v>
       </c>
       <c r="I8" t="n">
-        <v>132.95</v>
+        <v>132.949999999999989</v>
       </c>
       <c r="J8" t="n">
-        <v>187.32</v>
+        <v>187.319999999999993</v>
       </c>
       <c r="K8" t="n">
-        <v>241.49</v>
+        <v>241.490000000000009</v>
       </c>
       <c r="L8" t="n">
-        <v>304.73</v>
+        <v>304.730000000000018</v>
       </c>
       <c r="M8" t="n">
-        <v>377.74</v>
+        <v>377.740000000000009</v>
       </c>
       <c r="N8" t="n">
-        <v>148.23</v>
-      </c>
-    </row>
-    <row r="9">
+        <v>148.22999999999999</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14">
       <c r="A9" s="1" t="n">
         <v>7</v>
       </c>
@@ -785,43 +777,43 @@
         <v>12</v>
       </c>
       <c r="C9" t="n">
-        <v>0.11871</v>
+        <v>0.118710000000000004</v>
       </c>
       <c r="D9" t="n">
-        <v>5.45</v>
+        <v>5.45000000000000018</v>
       </c>
       <c r="E9" t="n">
-        <v>12.3</v>
+        <v>12.3000000000000007</v>
       </c>
       <c r="F9" t="n">
-        <v>20.73</v>
+        <v>20.7300000000000004</v>
       </c>
       <c r="G9" t="n">
-        <v>30.94</v>
+        <v>30.9400000000000013</v>
       </c>
       <c r="H9" t="n">
-        <v>43.14</v>
+        <v>43.1400000000000006</v>
       </c>
       <c r="I9" t="n">
         <v>57.5</v>
       </c>
       <c r="J9" t="n">
-        <v>80.65000000000001</v>
+        <v>80.6500000000000057</v>
       </c>
       <c r="K9" t="n">
-        <v>100.65</v>
+        <v>100.650000000000006</v>
       </c>
       <c r="L9" t="n">
-        <v>123.51</v>
+        <v>123.510000000000005</v>
       </c>
       <c r="M9" t="n">
-        <v>149.43</v>
+        <v>149.430000000000007</v>
       </c>
       <c r="N9" t="n">
-        <v>62.43</v>
-      </c>
-    </row>
-    <row r="10">
+        <v>62.4299999999999997</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14">
       <c r="A10" s="1" t="n">
         <v>8</v>
       </c>
@@ -829,43 +821,43 @@
         <v>13</v>
       </c>
       <c r="C10" t="n">
-        <v>0.13389</v>
+        <v>0.13389000000000002</v>
       </c>
       <c r="D10" t="n">
-        <v>4.41</v>
+        <v>4.41000000000000014</v>
       </c>
       <c r="E10" t="n">
-        <v>9.6</v>
+        <v>9.59999999999999964</v>
       </c>
       <c r="F10" t="n">
-        <v>15.65</v>
+        <v>15.6500000000000004</v>
       </c>
       <c r="G10" t="n">
-        <v>22.64</v>
+        <v>22.6400000000000006</v>
       </c>
       <c r="H10" t="n">
-        <v>30.67</v>
+        <v>30.6700000000000017</v>
       </c>
       <c r="I10" t="n">
-        <v>39.81</v>
+        <v>39.8100000000000023</v>
       </c>
       <c r="J10" t="n">
-        <v>55.69</v>
+        <v>55.6899999999999977</v>
       </c>
       <c r="K10" t="n">
         <v>67.75</v>
       </c>
       <c r="L10" t="n">
-        <v>81.23</v>
+        <v>81.230000000000004</v>
       </c>
       <c r="M10" t="n">
-        <v>96.22</v>
+        <v>96.2199999999999989</v>
       </c>
       <c r="N10" t="n">
-        <v>42.37</v>
-      </c>
-    </row>
-    <row r="11">
+        <v>42.3699999999999974</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14">
       <c r="A11" s="1" t="n">
         <v>9</v>
       </c>
@@ -873,43 +865,43 @@
         <v>14</v>
       </c>
       <c r="C11" t="n">
-        <v>0.097464</v>
+        <v>0.0974639999999999951</v>
       </c>
       <c r="D11" t="n">
-        <v>2.65</v>
+        <v>2.64999999999999991</v>
       </c>
       <c r="E11" t="n">
-        <v>5.29</v>
+        <v>5.29000000000000004</v>
       </c>
       <c r="F11" t="n">
-        <v>7.88</v>
+        <v>7.87999999999999989</v>
       </c>
       <c r="G11" t="n">
-        <v>10.4</v>
+        <v>10.4000000000000004</v>
       </c>
       <c r="H11" t="n">
-        <v>12.81</v>
+        <v>12.8100000000000005</v>
       </c>
       <c r="I11" t="n">
-        <v>15.09</v>
+        <v>15.0899999999999999</v>
       </c>
       <c r="J11" t="n">
-        <v>21.53</v>
+        <v>21.5300000000000011</v>
       </c>
       <c r="K11" t="n">
-        <v>23.52</v>
+        <v>23.5199999999999996</v>
       </c>
       <c r="L11" t="n">
-        <v>25.28</v>
+        <v>25.2800000000000011</v>
       </c>
       <c r="M11" t="n">
-        <v>26.78</v>
+        <v>26.7800000000000011</v>
       </c>
       <c r="N11" t="n">
-        <v>15.12</v>
-      </c>
-    </row>
-    <row r="12">
+        <v>15.1199999999999992</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14">
       <c r="A12" s="1" t="n">
         <v>10</v>
       </c>
@@ -917,43 +909,43 @@
         <v>15</v>
       </c>
       <c r="C12" t="n">
-        <v>0.09748900000000001</v>
+        <v>0.0974890000000000079</v>
       </c>
       <c r="D12" t="n">
-        <v>2.62</v>
+        <v>2.62000000000000011</v>
       </c>
       <c r="E12" t="n">
-        <v>5.21</v>
+        <v>5.20999999999999996</v>
       </c>
       <c r="F12" t="n">
-        <v>7.74</v>
+        <v>7.74000000000000021</v>
       </c>
       <c r="G12" t="n">
-        <v>10.17</v>
+        <v>10.1700000000000017</v>
       </c>
       <c r="H12" t="n">
-        <v>12.47</v>
+        <v>12.4700000000000006</v>
       </c>
       <c r="I12" t="n">
-        <v>14.61</v>
+        <v>14.6099999999999994</v>
       </c>
       <c r="J12" t="n">
-        <v>20.86</v>
+        <v>20.8599999999999994</v>
       </c>
       <c r="K12" t="n">
-        <v>22.65</v>
+        <v>22.6499999999999986</v>
       </c>
       <c r="L12" t="n">
-        <v>24.17</v>
+        <v>24.1700000000000017</v>
       </c>
       <c r="M12" t="n">
-        <v>25.4</v>
+        <v>25.3999999999999986</v>
       </c>
       <c r="N12" t="n">
-        <v>14.59</v>
-      </c>
-    </row>
-    <row r="13">
+        <v>14.5899999999999999</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14">
       <c r="A13" s="1" t="n">
         <v>11</v>
       </c>
@@ -961,43 +953,43 @@
         <v>16</v>
       </c>
       <c r="C13" t="n">
-        <v>0.14202</v>
+        <v>0.142020000000000017</v>
       </c>
       <c r="D13" t="n">
-        <v>3.62</v>
+        <v>3.62000000000000011</v>
       </c>
       <c r="E13" t="n">
-        <v>7.58</v>
+        <v>7.58000000000000007</v>
       </c>
       <c r="F13" t="n">
-        <v>11.9</v>
+        <v>11.9000000000000004</v>
       </c>
       <c r="G13" t="n">
-        <v>16.6</v>
+        <v>16.6000000000000014</v>
       </c>
       <c r="H13" t="n">
-        <v>21.68</v>
+        <v>21.6799999999999997</v>
       </c>
       <c r="I13" t="n">
-        <v>27.17</v>
+        <v>27.1700000000000017</v>
       </c>
       <c r="J13" t="n">
-        <v>37.99</v>
+        <v>37.990000000000002</v>
       </c>
       <c r="K13" t="n">
-        <v>44.56</v>
+        <v>44.5600000000000023</v>
       </c>
       <c r="L13" t="n">
-        <v>51.6</v>
+        <v>51.6000000000000014</v>
       </c>
       <c r="M13" t="n">
-        <v>59.12</v>
+        <v>59.1199999999999974</v>
       </c>
       <c r="N13" t="n">
-        <v>28.18</v>
-      </c>
-    </row>
-    <row r="14">
+        <v>28.1799999999999997</v>
+      </c>
+    </row>
+    <row r="14" spans="1:14">
       <c r="A14" s="1" t="n">
         <v>12</v>
       </c>
@@ -1005,43 +997,43 @@
         <v>17</v>
       </c>
       <c r="C14" t="n">
-        <v>0.33976</v>
+        <v>0.339760000000000018</v>
       </c>
       <c r="D14" t="n">
-        <v>0.98</v>
+        <v>0.980000000000000071</v>
       </c>
       <c r="E14" t="n">
         <v>1.25</v>
       </c>
       <c r="F14" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.689999999999999947</v>
       </c>
       <c r="G14" t="n">
-        <v>0.83</v>
+        <v>0.829999999999999893</v>
       </c>
       <c r="H14" t="n">
-        <v>3.42</v>
+        <v>3.41999999999999993</v>
       </c>
       <c r="I14" t="n">
-        <v>7.21</v>
+        <v>7.20999999999999996</v>
       </c>
       <c r="J14" t="n">
-        <v>9.08</v>
+        <v>9.08000000000000007</v>
       </c>
       <c r="K14" t="n">
-        <v>15.88</v>
+        <v>15.8800000000000008</v>
       </c>
       <c r="L14" t="n">
-        <v>24.29</v>
+        <v>24.2899999999999991</v>
       </c>
       <c r="M14" t="n">
-        <v>34.44</v>
+        <v>34.4399999999999977</v>
       </c>
       <c r="N14" t="n">
-        <v>9.81</v>
-      </c>
-    </row>
-    <row r="15">
+        <v>9.8100000000000005</v>
+      </c>
+    </row>
+    <row r="15" spans="1:14">
       <c r="A15" s="1" t="n">
         <v>13</v>
       </c>
@@ -1049,43 +1041,43 @@
         <v>18</v>
       </c>
       <c r="C15" t="n">
-        <v>0.26889</v>
+        <v>0.268890000000000029</v>
       </c>
       <c r="D15" t="n">
-        <v>3.97</v>
+        <v>3.97000000000000028</v>
       </c>
       <c r="E15" t="n">
-        <v>8.65</v>
+        <v>8.65000000000000036</v>
       </c>
       <c r="F15" t="n">
-        <v>14.12</v>
+        <v>14.1199999999999992</v>
       </c>
       <c r="G15" t="n">
-        <v>20.47</v>
+        <v>20.4699999999999989</v>
       </c>
       <c r="H15" t="n">
-        <v>27.79</v>
+        <v>27.7899999999999991</v>
       </c>
       <c r="I15" t="n">
-        <v>36.15</v>
+        <v>36.1499999999999986</v>
       </c>
       <c r="J15" t="n">
-        <v>51.02</v>
+        <v>51.0200000000000031</v>
       </c>
       <c r="K15" t="n">
-        <v>62.14</v>
+        <v>62.1400000000000006</v>
       </c>
       <c r="L15" t="n">
-        <v>74.59999999999999</v>
+        <v>74.5999999999999801</v>
       </c>
       <c r="M15" t="n">
-        <v>88.48999999999999</v>
+        <v>88.4899999999999807</v>
       </c>
       <c r="N15" t="n">
-        <v>38.74</v>
-      </c>
-    </row>
-    <row r="16">
+        <v>38.740000000000002</v>
+      </c>
+    </row>
+    <row r="16" spans="1:14">
       <c r="A16" s="1" t="n">
         <v>14</v>
       </c>
@@ -1093,43 +1085,43 @@
         <v>19</v>
       </c>
       <c r="C16" t="n">
-        <v>0.27845</v>
+        <v>0.278449999999999953</v>
       </c>
       <c r="D16" t="n">
-        <v>4.77</v>
+        <v>4.76999999999999957</v>
       </c>
       <c r="E16" t="n">
-        <v>10.45</v>
+        <v>10.4499999999999993</v>
       </c>
       <c r="F16" t="n">
-        <v>17.15</v>
+        <v>17.149999999999995</v>
       </c>
       <c r="G16" t="n">
-        <v>24.97</v>
+        <v>24.9699999999999989</v>
       </c>
       <c r="H16" t="n">
-        <v>34.01</v>
+        <v>34.009999999999998</v>
       </c>
       <c r="I16" t="n">
-        <v>44.36</v>
+        <v>44.3599999999999994</v>
       </c>
       <c r="J16" t="n">
-        <v>61.88</v>
+        <v>61.8800000000000026</v>
       </c>
       <c r="K16" t="n">
-        <v>75.65000000000001</v>
+        <v>75.6500000000000057</v>
       </c>
       <c r="L16" t="n">
-        <v>91.09999999999999</v>
+        <v>91.0999999999999943</v>
       </c>
       <c r="M16" t="n">
-        <v>108.32</v>
+        <v>108.319999999999993</v>
       </c>
       <c r="N16" t="n">
-        <v>47.27</v>
-      </c>
-    </row>
-    <row r="17">
+        <v>47.2700000000000031</v>
+      </c>
+    </row>
+    <row r="17" spans="1:14">
       <c r="A17" s="1" t="n">
         <v>15</v>
       </c>
@@ -1137,43 +1129,43 @@
         <v>20</v>
       </c>
       <c r="C17" t="n">
-        <v>0.31894</v>
+        <v>0.318940000000000001</v>
       </c>
       <c r="D17" t="n">
-        <v>4.76</v>
+        <v>4.75999999999999979</v>
       </c>
       <c r="E17" t="n">
-        <v>10.39</v>
+        <v>10.3900000000000006</v>
       </c>
       <c r="F17" t="n">
-        <v>16.98</v>
+        <v>16.9800000000000004</v>
       </c>
       <c r="G17" t="n">
-        <v>24.61</v>
+        <v>24.6099999999999994</v>
       </c>
       <c r="H17" t="n">
-        <v>33.38</v>
+        <v>33.3800000000000026</v>
       </c>
       <c r="I17" t="n">
-        <v>43.37</v>
+        <v>43.3699999999999974</v>
       </c>
       <c r="J17" t="n">
-        <v>60.38</v>
+        <v>60.3800000000000026</v>
       </c>
       <c r="K17" t="n">
-        <v>73.56</v>
+        <v>73.5600000000000023</v>
       </c>
       <c r="L17" t="n">
-        <v>88.29000000000001</v>
+        <v>88.2900000000000063</v>
       </c>
       <c r="M17" t="n">
-        <v>104.66</v>
+        <v>104.659999999999997</v>
       </c>
       <c r="N17" t="n">
-        <v>46.04</v>
-      </c>
-    </row>
-    <row r="18">
+        <v>46.0399999999999991</v>
+      </c>
+    </row>
+    <row r="18" spans="1:14">
       <c r="A18" s="1" t="n">
         <v>16</v>
       </c>
@@ -1181,43 +1173,43 @@
         <v>21</v>
       </c>
       <c r="C18" t="n">
-        <v>0.34913</v>
+        <v>0.349129999999999985</v>
       </c>
       <c r="D18" t="n">
-        <v>2.12</v>
+        <v>2.12000000000000011</v>
       </c>
       <c r="E18" t="n">
-        <v>4.16</v>
+        <v>4.16000000000000014</v>
       </c>
       <c r="F18" t="n">
-        <v>6.12</v>
+        <v>6.12000000000000011</v>
       </c>
       <c r="G18" t="n">
-        <v>7.97</v>
+        <v>7.96999999999999886</v>
       </c>
       <c r="H18" t="n">
-        <v>9.73</v>
+        <v>9.73000000000000043</v>
       </c>
       <c r="I18" t="n">
-        <v>11.37</v>
+        <v>11.3699999999999992</v>
       </c>
       <c r="J18" t="n">
-        <v>17.04</v>
+        <v>17.0399999999999991</v>
       </c>
       <c r="K18" t="n">
-        <v>18.47</v>
+        <v>18.4699999999999989</v>
       </c>
       <c r="L18" t="n">
         <v>19.75</v>
       </c>
       <c r="M18" t="n">
-        <v>20.87</v>
+        <v>20.870000000000001</v>
       </c>
       <c r="N18" t="n">
-        <v>11.76</v>
-      </c>
-    </row>
-    <row r="19">
+        <v>11.7599999999999998</v>
+      </c>
+    </row>
+    <row r="19" spans="1:14">
       <c r="A19" s="1" t="n">
         <v>17</v>
       </c>
@@ -1225,43 +1217,43 @@
         <v>22</v>
       </c>
       <c r="C19" t="n">
-        <v>0.36302</v>
+        <v>0.363020000000000032</v>
       </c>
       <c r="D19" t="n">
-        <v>1.82</v>
+        <v>1.82000000000000011</v>
       </c>
       <c r="E19" t="n">
-        <v>3.46</v>
+        <v>3.45999999999999996</v>
       </c>
       <c r="F19" t="n">
-        <v>4.9</v>
+        <v>4.90000000000000036</v>
       </c>
       <c r="G19" t="n">
-        <v>6.1</v>
+        <v>6.09999999999999964</v>
       </c>
       <c r="H19" t="n">
-        <v>7.06</v>
+        <v>7.05999999999999961</v>
       </c>
       <c r="I19" t="n">
         <v>7.75</v>
       </c>
       <c r="J19" t="n">
-        <v>12.14</v>
+        <v>12.1400000000000006</v>
       </c>
       <c r="K19" t="n">
-        <v>12.23</v>
+        <v>12.2300000000000004</v>
       </c>
       <c r="L19" t="n">
-        <v>11.97</v>
+        <v>11.9700000000000006</v>
       </c>
       <c r="M19" t="n">
-        <v>11.35</v>
+        <v>11.3499999999999996</v>
       </c>
       <c r="N19" t="n">
-        <v>7.88</v>
-      </c>
-    </row>
-    <row r="20">
+        <v>7.87999999999999989</v>
+      </c>
+    </row>
+    <row r="20" spans="1:14">
       <c r="A20" s="1" t="n">
         <v>18</v>
       </c>
@@ -1269,43 +1261,43 @@
         <v>23</v>
       </c>
       <c r="C20" t="n">
-        <v>0.46354</v>
+        <v>0.463539999999999974</v>
       </c>
       <c r="D20" t="n">
-        <v>2.08</v>
+        <v>2.08000000000000007</v>
       </c>
       <c r="E20" t="n">
-        <v>4.1</v>
+        <v>4.09999999999999964</v>
       </c>
       <c r="F20" t="n">
-        <v>6.03</v>
+        <v>6.03000000000000025</v>
       </c>
       <c r="G20" t="n">
-        <v>7.87</v>
+        <v>7.87000000000000011</v>
       </c>
       <c r="H20" t="n">
-        <v>9.6</v>
+        <v>9.59999999999999964</v>
       </c>
       <c r="I20" t="n">
-        <v>11.23</v>
+        <v>11.2300000000000004</v>
       </c>
       <c r="J20" t="n">
-        <v>16.9</v>
+        <v>16.899999999999995</v>
       </c>
       <c r="K20" t="n">
-        <v>18.33</v>
+        <v>18.3299999999999983</v>
       </c>
       <c r="L20" t="n">
-        <v>19.62</v>
+        <v>19.620000000000001</v>
       </c>
       <c r="M20" t="n">
         <v>20.75</v>
       </c>
       <c r="N20" t="n">
-        <v>11.65</v>
-      </c>
-    </row>
-    <row r="21">
+        <v>11.6500000000000004</v>
+      </c>
+    </row>
+    <row r="21" spans="1:14">
       <c r="A21" s="1" t="n">
         <v>19</v>
       </c>
@@ -1313,43 +1305,43 @@
         <v>24</v>
       </c>
       <c r="C21" t="n">
-        <v>0.43849</v>
+        <v>0.438490000000000002</v>
       </c>
       <c r="D21" t="n">
         <v>3</v>
       </c>
       <c r="E21" t="n">
-        <v>6.32</v>
+        <v>6.32000000000000028</v>
       </c>
       <c r="F21" t="n">
-        <v>9.970000000000001</v>
+        <v>9.97000000000000064</v>
       </c>
       <c r="G21" t="n">
         <v>14</v>
       </c>
       <c r="H21" t="n">
-        <v>18.44</v>
+        <v>18.4400000000000013</v>
       </c>
       <c r="I21" t="n">
-        <v>23.32</v>
+        <v>23.3200000000000003</v>
       </c>
       <c r="J21" t="n">
-        <v>33.42</v>
+        <v>33.4200000000000017</v>
       </c>
       <c r="K21" t="n">
         <v>39.5</v>
       </c>
       <c r="L21" t="n">
-        <v>46.14</v>
+        <v>46.1400000000000006</v>
       </c>
       <c r="M21" t="n">
-        <v>53.38</v>
+        <v>53.3800000000000026</v>
       </c>
       <c r="N21" t="n">
         <v>24.75</v>
       </c>
     </row>
-    <row r="22">
+    <row r="22" spans="1:14">
       <c r="A22" s="1" t="n">
         <v>20</v>
       </c>
@@ -1357,43 +1349,43 @@
         <v>25</v>
       </c>
       <c r="C22" t="n">
-        <v>0.45643</v>
+        <v>0.456430000000000025</v>
       </c>
       <c r="D22" t="n">
-        <v>3.43</v>
+        <v>3.43000000000000016</v>
       </c>
       <c r="E22" t="n">
-        <v>7.27</v>
+        <v>7.26999999999999869</v>
       </c>
       <c r="F22" t="n">
-        <v>11.56</v>
+        <v>11.5600000000000005</v>
       </c>
       <c r="G22" t="n">
-        <v>16.33</v>
+        <v>16.3299999999999983</v>
       </c>
       <c r="H22" t="n">
-        <v>21.64</v>
+        <v>21.6400000000000006</v>
       </c>
       <c r="I22" t="n">
-        <v>27.51</v>
+        <v>27.5100000000000016</v>
       </c>
       <c r="J22" t="n">
-        <v>38.93</v>
+        <v>38.9299999999999997</v>
       </c>
       <c r="K22" t="n">
-        <v>46.31</v>
+        <v>46.3100000000000023</v>
       </c>
       <c r="L22" t="n">
-        <v>54.41</v>
+        <v>54.4099999999999966</v>
       </c>
       <c r="M22" t="n">
-        <v>63.26</v>
+        <v>63.259999999999998</v>
       </c>
       <c r="N22" t="n">
-        <v>29.06</v>
-      </c>
-    </row>
-    <row r="23">
+        <v>29.0599999999999987</v>
+      </c>
+    </row>
+    <row r="23" spans="1:14">
       <c r="A23" s="1" t="n">
         <v>21</v>
       </c>
@@ -1401,43 +1393,43 @@
         <v>26</v>
       </c>
       <c r="C23" t="n">
-        <v>0.5197000000000001</v>
+        <v>0.519700000000000095</v>
       </c>
       <c r="D23" t="n">
-        <v>2.91</v>
+        <v>2.91000000000000014</v>
       </c>
       <c r="E23" t="n">
-        <v>6.06</v>
+        <v>6.05999999999999961</v>
       </c>
       <c r="F23" t="n">
-        <v>9.470000000000001</v>
+        <v>9.47000000000000064</v>
       </c>
       <c r="G23" t="n">
-        <v>13.16</v>
+        <v>13.1600000000000001</v>
       </c>
       <c r="H23" t="n">
-        <v>17.14</v>
+        <v>17.1400000000000006</v>
       </c>
       <c r="I23" t="n">
-        <v>21.45</v>
+        <v>21.4499999999999993</v>
       </c>
       <c r="J23" t="n">
-        <v>30.76</v>
+        <v>30.7600000000000016</v>
       </c>
       <c r="K23" t="n">
-        <v>35.97</v>
+        <v>35.9699999999999989</v>
       </c>
       <c r="L23" t="n">
-        <v>41.59</v>
+        <v>41.5900000000000034</v>
       </c>
       <c r="M23" t="n">
-        <v>47.63</v>
+        <v>47.6300000000000026</v>
       </c>
       <c r="N23" t="n">
-        <v>22.62</v>
-      </c>
-    </row>
-    <row r="24">
+        <v>22.620000000000001</v>
+      </c>
+    </row>
+    <row r="24" spans="1:14">
       <c r="A24" s="1" t="n">
         <v>22</v>
       </c>
@@ -1445,43 +1437,43 @@
         <v>27</v>
       </c>
       <c r="C24" t="n">
-        <v>0.57867</v>
+        <v>0.578669999999999973</v>
       </c>
       <c r="D24" t="n">
-        <v>2.14</v>
+        <v>2.14000000000000012</v>
       </c>
       <c r="E24" t="n">
-        <v>4.27</v>
+        <v>4.26999999999999957</v>
       </c>
       <c r="F24" t="n">
-        <v>6.39</v>
+        <v>6.38999999999999968</v>
       </c>
       <c r="G24" t="n">
         <v>8.5</v>
       </c>
       <c r="H24" t="n">
-        <v>10.6</v>
+        <v>10.5999999999999996</v>
       </c>
       <c r="I24" t="n">
-        <v>12.7</v>
+        <v>12.6999999999999993</v>
       </c>
       <c r="J24" t="n">
-        <v>19.02</v>
+        <v>19.0199999999999996</v>
       </c>
       <c r="K24" t="n">
-        <v>21.18</v>
+        <v>21.1799999999999997</v>
       </c>
       <c r="L24" t="n">
-        <v>23.34</v>
+        <v>23.3399999999999999</v>
       </c>
       <c r="M24" t="n">
         <v>25.5</v>
       </c>
       <c r="N24" t="n">
-        <v>13.36</v>
-      </c>
-    </row>
-    <row r="25">
+        <v>13.3599999999999994</v>
+      </c>
+    </row>
+    <row r="25" spans="1:14">
       <c r="A25" s="1" t="n">
         <v>23</v>
       </c>
@@ -1489,43 +1481,43 @@
         <v>28</v>
       </c>
       <c r="C25" t="n">
-        <v>0.51812</v>
+        <v>0.518120000000000047</v>
       </c>
       <c r="D25" t="n">
         <v>2</v>
       </c>
       <c r="E25" t="n">
-        <v>3.92</v>
+        <v>3.91999999999999993</v>
       </c>
       <c r="F25" t="n">
-        <v>5.76</v>
+        <v>5.75999999999999979</v>
       </c>
       <c r="G25" t="n">
-        <v>7.51</v>
+        <v>7.5099999999999989</v>
       </c>
       <c r="H25" t="n">
-        <v>9.17</v>
+        <v>9.17000000000000171</v>
       </c>
       <c r="I25" t="n">
-        <v>10.73</v>
+        <v>10.7300000000000004</v>
       </c>
       <c r="J25" t="n">
-        <v>16.32</v>
+        <v>16.3200000000000003</v>
       </c>
       <c r="K25" t="n">
-        <v>17.71</v>
+        <v>17.7100000000000009</v>
       </c>
       <c r="L25" t="n">
-        <v>18.98</v>
+        <v>18.9800000000000004</v>
       </c>
       <c r="M25" t="n">
-        <v>20.13</v>
+        <v>20.129999999999999</v>
       </c>
       <c r="N25" t="n">
-        <v>11.22</v>
-      </c>
-    </row>
-    <row r="26">
+        <v>11.2200000000000006</v>
+      </c>
+    </row>
+    <row r="26" spans="1:14">
       <c r="A26" s="1" t="n">
         <v>24</v>
       </c>
@@ -1533,43 +1525,43 @@
         <v>29</v>
       </c>
       <c r="C26" t="n">
-        <v>0.5415</v>
+        <v>0.541500000000000004</v>
       </c>
       <c r="D26" t="n">
-        <v>1.82</v>
+        <v>1.82000000000000011</v>
       </c>
       <c r="E26" t="n">
-        <v>3.51</v>
+        <v>3.50999999999999979</v>
       </c>
       <c r="F26" t="n">
-        <v>5.06</v>
+        <v>5.05999999999999961</v>
       </c>
       <c r="G26" t="n">
-        <v>6.47</v>
+        <v>6.46999999999999975</v>
       </c>
       <c r="H26" t="n">
-        <v>7.72</v>
+        <v>7.71999999999999886</v>
       </c>
       <c r="I26" t="n">
-        <v>8.800000000000001</v>
+        <v>8.80000000000000071</v>
       </c>
       <c r="J26" t="n">
-        <v>13.76</v>
+        <v>13.7599999999999998</v>
       </c>
       <c r="K26" t="n">
         <v>14.5</v>
       </c>
       <c r="L26" t="n">
-        <v>15.05</v>
+        <v>15.0500000000000007</v>
       </c>
       <c r="M26" t="n">
-        <v>15.37</v>
+        <v>15.3699999999999992</v>
       </c>
       <c r="N26" t="n">
-        <v>9.210000000000001</v>
-      </c>
-    </row>
-    <row r="27">
+        <v>9.21000000000000085</v>
+      </c>
+    </row>
+    <row r="27" spans="1:14">
       <c r="A27" s="1" t="n">
         <v>25</v>
       </c>
@@ -1577,43 +1569,69 @@
         <v>30</v>
       </c>
       <c r="C27" t="n">
-        <v>0.55535</v>
+        <v>0.555349999999999966</v>
       </c>
       <c r="D27" t="n">
         <v>1.95</v>
       </c>
       <c r="E27" t="n">
-        <v>3.8</v>
+        <v>3.79999999999999982</v>
       </c>
       <c r="F27" t="n">
-        <v>5.56</v>
+        <v>5.55999999999999961</v>
       </c>
       <c r="G27" t="n">
-        <v>7.21</v>
+        <v>7.20999999999999996</v>
       </c>
       <c r="H27" t="n">
         <v>8.75</v>
       </c>
       <c r="I27" t="n">
-        <v>10.16</v>
+        <v>10.1600000000000001</v>
       </c>
       <c r="J27" t="n">
-        <v>15.56</v>
+        <v>15.5600000000000005</v>
       </c>
       <c r="K27" t="n">
-        <v>16.76</v>
+        <v>16.7600000000000016</v>
       </c>
       <c r="L27" t="n">
-        <v>17.81</v>
+        <v>17.8099999999999952</v>
       </c>
       <c r="M27" t="n">
-        <v>18.71</v>
+        <v>18.7100000000000009</v>
       </c>
       <c r="N27" t="n">
-        <v>10.63</v>
+        <v>10.6300000000000008</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <printOptions>
+    <extLst>
+      <ext uri="smNativeData">
+        <pm:pageFlags xmlns:pm="smNativeData" id="1699202731" printRowHead="0" printColHead="0" printHeadLine="0" printFootLine="0" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+      </ext>
+    </extLst>
+  </printOptions>
+  <pageMargins left="0.750000" right="0.750000" top="1.000000" bottom="1.000000" header="0.500000" footer="0.500000"/>
+  <pageSetup paperSize="1" fitToWidth="0" fitToHeight="1" pageOrder="overThenDown"/>
+  <headerFooter>
+    <extLst>
+      <ext uri="smNativeData">
+        <pm:header xmlns:pm="smNativeData" id="1699202731" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1699202731" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:paperBin xmlns:pm="smNativeData" id="1699202731" Id="0" type="0" value="0"/>
+        <pm:paperBin xmlns:pm="smNativeData" id="1699202731" Id="1" type="0" value="0"/>
+      </ext>
+    </extLst>
+  </headerFooter>
+  <extLst>
+    <ext uri="smNativeData">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1699202731" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+        <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
+        <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
+      </pm:sheetPrefs>
+    </ext>
+  </extLst>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Updated on 11-05-2023 at 17:21
</commit_message>
<xml_diff>
--- a/output/accuracy_cubic.xlsx
+++ b/output/accuracy_cubic.xlsx
@@ -13,10 +13,10 @@
   <calcPr/>
   <extLst>
     <ext uri="smNativeData">
-      <pm:revision xmlns:pm="smNativeData" day="1699202731" val="1066" rev="124" revOS="4" revMin="124" revMax="0"/>
-      <pm:docPrefs xmlns:pm="smNativeData" id="1699202731" fixedDigits="0" showNotice="1" showFrameBounds="1" autoChart="1" recalcOnPrint="1" recalcOnCopy="1" finalRounding="1" compatTextArt="1" tab="567" useDefinedPrintRange="1" printArea="currentSheet"/>
-      <pm:compatibility xmlns:pm="smNativeData" id="1699202731" overlapCells="1"/>
-      <pm:defCurrency xmlns:pm="smNativeData" id="1699202731"/>
+      <pm:revision xmlns:pm="smNativeData" day="1699203626" val="1066" rev="124" revOS="4" revMin="124" revMax="0"/>
+      <pm:docPrefs xmlns:pm="smNativeData" id="1699203626" fixedDigits="0" showNotice="1" showFrameBounds="1" autoChart="1" recalcOnPrint="1" recalcOnCopy="1" finalRounding="1" compatTextArt="1" tab="567" useDefinedPrintRange="1" printArea="currentSheet"/>
+      <pm:compatibility xmlns:pm="smNativeData" id="1699203626" overlapCells="1"/>
+      <pm:defCurrency xmlns:pm="smNativeData" id="1699203626"/>
     </ext>
   </extLst>
 </workbook>
@@ -42,7 +42,7 @@
       <sz val="11"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1699202731" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1699203626" ulstyle="none" kern="1">
             <pm:latin face="Calibri" sz="220" lang="default"/>
             <pm:cs face="Times New Roman" sz="220" lang="default"/>
             <pm:ea face="SimSun" sz="220" lang="default"/>
@@ -57,7 +57,7 @@
       <sz val="10"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1699202731" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1699203626" ulstyle="none" kern="1">
             <pm:latin face="Arial" sz="200" lang="default"/>
             <pm:cs face="Times New Roman" sz="200" lang="default"/>
             <pm:ea face="SimSun" sz="200" lang="default"/>
@@ -73,7 +73,7 @@
       <sz val="10"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1699202731" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1699203626" ulstyle="none" kern="1">
             <pm:latin face="Arial" sz="200" lang="default" weight="bold"/>
             <pm:cs face="Times New Roman" sz="200" lang="default" weight="bold"/>
             <pm:ea face="SimSun" sz="200" lang="default" weight="bold"/>
@@ -109,7 +109,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1699202731"/>
+          <pm:border xmlns:pm="smNativeData" id="1699203626"/>
         </ext>
       </extLst>
     </border>
@@ -128,7 +128,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1699202731">
+          <pm:border xmlns:pm="smNativeData" id="1699203626">
             <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
@@ -150,12 +150,17 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" customBuiltin="1"/>
   </cellStyles>
+  <dxfs count="1"/>
   <tableStyles count="0"/>
   <extLst>
     <ext uri="smNativeData">
-      <pm:charStyles xmlns:pm="smNativeData" id="1699202731" count="1">
+      <pm:charStyles xmlns:pm="smNativeData" id="1699203626" count="1">
         <pm:charStyle name="Normal" fontId="0" Id="1"/>
       </pm:charStyles>
+      <pm:colors xmlns:pm="smNativeData" id="1699203626" count="2">
+        <pm:color name="azul2" rgb="3E76C1"/>
+        <pm:color name="naranja" rgb="F36F0C"/>
+      </pm:colors>
     </ext>
   </extLst>
 </styleSheet>
@@ -540,7 +545,7 @@
         <v>754.129999999999995</v>
       </c>
       <c r="L3" t="n">
-        <v>982.380000000000109</v>
+        <v>982.379999999999995</v>
       </c>
       <c r="M3" t="n">
         <v>1251.81999999999994</v>
@@ -921,7 +926,7 @@
         <v>7.74000000000000021</v>
       </c>
       <c r="G12" t="n">
-        <v>10.1700000000000017</v>
+        <v>10.1699999999999999</v>
       </c>
       <c r="H12" t="n">
         <v>12.4700000000000006</v>
@@ -1185,7 +1190,7 @@
         <v>6.12000000000000011</v>
       </c>
       <c r="G18" t="n">
-        <v>7.96999999999999886</v>
+        <v>7.96999999999999975</v>
       </c>
       <c r="H18" t="n">
         <v>9.73000000000000043</v>
@@ -1493,10 +1498,10 @@
         <v>5.75999999999999979</v>
       </c>
       <c r="G25" t="n">
-        <v>7.5099999999999989</v>
+        <v>7.50999999999999979</v>
       </c>
       <c r="H25" t="n">
-        <v>9.17000000000000171</v>
+        <v>9.16999999999999993</v>
       </c>
       <c r="I25" t="n">
         <v>10.7300000000000004</v>
@@ -1540,7 +1545,7 @@
         <v>6.46999999999999975</v>
       </c>
       <c r="H26" t="n">
-        <v>7.71999999999999886</v>
+        <v>7.71999999999999975</v>
       </c>
       <c r="I26" t="n">
         <v>8.80000000000000071</v>
@@ -1606,10 +1611,22 @@
       </c>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="D2:M27">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="20"/>
+        <cfvo type="num" val="100"/>
+        <color rgb="FF3E76C1"/>
+        <color rgb="FFF36F0C"/>
+        <color rgb="FFFF0000"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1699202731" printRowHead="0" printColHead="0" printHeadLine="0" printFootLine="0" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1699203626" printRowHead="0" printColHead="0" printHeadLine="0" printFootLine="0" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -1618,16 +1635,16 @@
   <headerFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1699202731" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1699202731" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
-        <pm:paperBin xmlns:pm="smNativeData" id="1699202731" Id="0" type="0" value="0"/>
-        <pm:paperBin xmlns:pm="smNativeData" id="1699202731" Id="1" type="0" value="0"/>
+        <pm:header xmlns:pm="smNativeData" id="1699203626" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1699203626" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:paperBin xmlns:pm="smNativeData" id="1699203626" Id="0" type="0" value="0"/>
+        <pm:paperBin xmlns:pm="smNativeData" id="1699203626" Id="1" type="0" value="0"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1699202731" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1699203626" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>

</xml_diff>

<commit_message>
Updated on 11-05-2023 at 22:29
</commit_message>
<xml_diff>
--- a/output/accuracy_cubic.xlsx
+++ b/output/accuracy_cubic.xlsx
@@ -1,168 +1,138 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4506"/>
-  <fileSharing readOnlyRecommended="0" userName="Gustavo"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
+  <workbookProtection/>
   <bookViews>
-    <workbookView activeTab="0" xWindow="240" yWindow="60" windowWidth="0" windowHeight="0" tabRatio="500"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr/>
-  <extLst>
-    <ext uri="smNativeData">
-      <pm:revision xmlns:pm="smNativeData" day="1699203626" val="1066" rev="124" revOS="4" revMin="124" revMax="0"/>
-      <pm:docPrefs xmlns:pm="smNativeData" id="1699203626" fixedDigits="0" showNotice="1" showFrameBounds="1" autoChart="1" recalcOnPrint="1" recalcOnCopy="1" finalRounding="1" compatTextArt="1" tab="567" useDefinedPrintRange="1" printArea="currentSheet"/>
-      <pm:compatibility xmlns:pm="smNativeData" id="1699203626" overlapCells="1"/>
-      <pm:defCurrency xmlns:pm="smNativeData" id="1699203626"/>
-    </ext>
-  </extLst>
+  <definedNames/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="8">
-    <numFmt numFmtId="5" formatCode="#,##0\ &quot;$&quot;;\-#,##0\ &quot;$&quot;"/>
-    <numFmt numFmtId="6" formatCode="#,##0\ &quot;$&quot;;[Red]\-#,##0\ &quot;$&quot;"/>
-    <numFmt numFmtId="7" formatCode="#,##0.00\ &quot;$&quot;;\-#,##0.00\ &quot;$&quot;"/>
-    <numFmt numFmtId="8" formatCode="#,##0.00\ &quot;$&quot;;[Red]\-#,##0.00\ &quot;$&quot;"/>
-    <numFmt numFmtId="42" formatCode="_-* #,##0\ &quot;$&quot;_-;\-* #,##0\ &quot;$&quot;_-;_-* &quot;-&quot;\ &quot;$&quot;_-;_-@_-"/>
-    <numFmt numFmtId="41" formatCode="_-* #,##0\ _$_-;\-* #,##0\ _$_-;_-* &quot;-&quot;\ _$_-;_-@_-"/>
-    <numFmt numFmtId="44" formatCode="_-* #,##0.00\ &quot;$&quot;_-;\-* #,##0.00\ &quot;$&quot;_-;_-* &quot;-&quot;??\ &quot;$&quot;_-;_-@_-"/>
-    <numFmt numFmtId="43" formatCode="_-* #,##0.00\ _$_-;\-* #,##0.00\ _$_-;_-* &quot;-&quot;??\ _$_-;_-@_-"/>
-  </numFmts>
-  <fonts count="3">
+  <numFmts count="0"/>
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
-      <color rgb="FF000000"/>
+      <color theme="1"/>
       <sz val="11"/>
-      <extLst>
-        <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1699203626" ulstyle="none" kern="1">
-            <pm:latin face="Calibri" sz="220" lang="default"/>
-            <pm:cs face="Times New Roman" sz="220" lang="default"/>
-            <pm:ea face="SimSun" sz="220" lang="default"/>
-          </pm:charSpec>
-        </ext>
-      </extLst>
+      <scheme val="minor"/>
     </font>
     <font>
-      <name val="Arial"/>
-      <family val="2"/>
-      <color rgb="FF000000"/>
-      <sz val="10"/>
-      <extLst>
-        <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1699203626" ulstyle="none" kern="1">
-            <pm:latin face="Arial" sz="200" lang="default"/>
-            <pm:cs face="Times New Roman" sz="200" lang="default"/>
-            <pm:ea face="SimSun" sz="200" lang="default"/>
-          </pm:charSpec>
-        </ext>
-      </extLst>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <family val="2"/>
-      <b/>
-      <color rgb="FF000000"/>
-      <sz val="10"/>
-      <extLst>
-        <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1699203626" ulstyle="none" kern="1">
-            <pm:latin face="Arial" sz="200" lang="default" weight="bold"/>
-            <pm:cs face="Times New Roman" sz="200" lang="default" weight="bold"/>
-            <pm:ea face="SimSun" sz="200" lang="default" weight="bold"/>
-          </pm:charSpec>
-        </ext>
-      </extLst>
+      <b val="1"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
-    <fill>
-      <patternFill patternType="none"/>
-    </fill>
   </fills>
   <borders count="2">
     <border>
-      <left style="none">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="none">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="none">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="none">
-        <color rgb="FF000000"/>
-      </bottom>
-      <extLst>
-        <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1699203626"/>
-        </ext>
-      </extLst>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <extLst>
-        <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1699203626">
-            <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
-            <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
-            <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
-            <pm:line position="right" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
-          </pm:border>
-        </ext>
-      </extLst>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" customBuiltin="1"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="1"/>
-  <tableStyles count="0"/>
-  <extLst>
-    <ext uri="smNativeData">
-      <pm:charStyles xmlns:pm="smNativeData" id="1699203626" count="1">
-        <pm:charStyle name="Normal" fontId="0" Id="1"/>
-      </pm:charStyles>
-      <pm:colors xmlns:pm="smNativeData" id="1699203626" count="2">
-        <pm:color name="azul2" rgb="3E76C1"/>
-        <pm:color name="naranja" rgb="F36F0C"/>
-      </pm:colors>
-    </ext>
-  </extLst>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -177,10 +147,10 @@
         <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="EEECE1"/>
+        <a:srgbClr val="1F497D"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="1F497D"/>
+        <a:srgbClr val="EEECE1"/>
       </a:lt2>
       <a:accent1>
         <a:srgbClr val="4F81BD"/>
@@ -212,11 +182,69 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
-        <a:ea typeface="SimSun"/>
-        <a:cs typeface="Times New Roman"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -386,46 +414,21 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults>
-    <a:spDef>
-      <a:spPr/>
-      <a:bodyPr>
-        <a:prstTxWarp prst="textNoShape">
-          <a:avLst/>
-        </a:prstTxWarp>
-        <a:noAutofit/>
-      </a:bodyPr>
-      <a:lstStyle>
-        <a:defPPr>
-          <a:defRPr/>
-        </a:defPPr>
-      </a:lstStyle>
-      <a:style>
-        <a:lnRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="lt1"/>
-        </a:fontRef>
-      </a:style>
-    </a:spDef>
-  </a:objectDefaults>
+  <a:objectDefaults/>
   <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:N27"/>
-  <sheetFormatPr defaultRowHeight="15.40"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="2:14">
+    <row r="1">
       <c r="B1" s="1" t="n">
         <v>0</v>
       </c>
@@ -466,7 +469,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:14">
+    <row r="2">
       <c r="A2" s="1" t="n">
         <v>0</v>
       </c>
@@ -474,43 +477,43 @@
         <v>5</v>
       </c>
       <c r="C2" t="n">
-        <v>0.0026476999999999995</v>
+        <v>0.0028902</v>
       </c>
       <c r="D2" t="n">
-        <v>25.3299999999999983</v>
+        <v>0.39</v>
       </c>
       <c r="E2" t="n">
-        <v>71.019999999999996</v>
+        <v>1.13</v>
       </c>
       <c r="F2" t="n">
-        <v>142.759999999999991</v>
+        <v>5.81</v>
       </c>
       <c r="G2" t="n">
-        <v>246.22999999999999</v>
+        <v>21.29</v>
       </c>
       <c r="H2" t="n">
-        <v>387.129999999999995</v>
+        <v>42.15</v>
       </c>
       <c r="I2" t="n">
-        <v>571.129999999999995</v>
+        <v>68.61</v>
       </c>
       <c r="J2" t="n">
-        <v>837.269999999999982</v>
+        <v>100.42</v>
       </c>
       <c r="K2" t="n">
-        <v>1135.16000000000008</v>
+        <v>142.17</v>
       </c>
       <c r="L2" t="n">
-        <v>1495.45000000000005</v>
+        <v>193.58</v>
       </c>
       <c r="M2" t="n">
-        <v>1924.02999999999997</v>
+        <v>255.32</v>
       </c>
       <c r="N2" t="n">
-        <v>683.549999999999955</v>
-      </c>
-    </row>
-    <row r="3" spans="1:14">
+        <v>83.09</v>
+      </c>
+    </row>
+    <row r="3">
       <c r="A3" s="1" t="n">
         <v>1</v>
       </c>
@@ -518,43 +521,43 @@
         <v>6</v>
       </c>
       <c r="C3" t="n">
-        <v>0.00753860000000000063</v>
+        <v>0.0043706</v>
       </c>
       <c r="D3" t="n">
-        <v>20.129999999999999</v>
+        <v>2.69</v>
       </c>
       <c r="E3" t="n">
-        <v>53.8200000000000003</v>
+        <v>9.42</v>
       </c>
       <c r="F3" t="n">
-        <v>104.329999999999998</v>
+        <v>18.5</v>
       </c>
       <c r="G3" t="n">
-        <v>174.939999999999998</v>
+        <v>22.42</v>
       </c>
       <c r="H3" t="n">
-        <v>268.920000000000016</v>
+        <v>27.73</v>
       </c>
       <c r="I3" t="n">
-        <v>389.54000000000002</v>
+        <v>34.19</v>
       </c>
       <c r="J3" t="n">
-        <v>563.659999999999968</v>
+        <v>51.61</v>
       </c>
       <c r="K3" t="n">
-        <v>754.129999999999995</v>
+        <v>71.31</v>
       </c>
       <c r="L3" t="n">
-        <v>982.379999999999995</v>
+        <v>92.25</v>
       </c>
       <c r="M3" t="n">
-        <v>1251.81999999999994</v>
+        <v>116.48</v>
       </c>
       <c r="N3" t="n">
-        <v>456.370000000000005</v>
-      </c>
-    </row>
-    <row r="4" spans="1:14">
+        <v>44.66</v>
+      </c>
+    </row>
+    <row r="4">
       <c r="A4" s="1" t="n">
         <v>2</v>
       </c>
@@ -565,40 +568,40 @@
         <v>0</v>
       </c>
       <c r="D4" t="n">
-        <v>0.560000000000000053</v>
+        <v>0.8</v>
       </c>
       <c r="E4" t="n">
-        <v>2.62999999999999989</v>
+        <v>5.92</v>
       </c>
       <c r="F4" t="n">
-        <v>7.33999999999999986</v>
+        <v>14.76</v>
       </c>
       <c r="G4" t="n">
-        <v>15.8100000000000005</v>
+        <v>21.07</v>
       </c>
       <c r="H4" t="n">
-        <v>29.1700000000000017</v>
+        <v>31.9</v>
       </c>
       <c r="I4" t="n">
-        <v>48.5499999999999972</v>
+        <v>47.49</v>
       </c>
       <c r="J4" t="n">
-        <v>81.5400000000000063</v>
+        <v>79.68000000000001</v>
       </c>
       <c r="K4" t="n">
-        <v>117.640000000000001</v>
+        <v>120.31</v>
       </c>
       <c r="L4" t="n">
-        <v>163.490000000000009</v>
+        <v>168.51</v>
       </c>
       <c r="M4" t="n">
-        <v>220.27000000000001</v>
+        <v>227.37</v>
       </c>
       <c r="N4" t="n">
-        <v>68.7000000000000028</v>
-      </c>
-    </row>
-    <row r="5" spans="1:14">
+        <v>71.78</v>
+      </c>
+    </row>
+    <row r="5">
       <c r="A5" s="1" t="n">
         <v>3</v>
       </c>
@@ -606,43 +609,43 @@
         <v>8</v>
       </c>
       <c r="C5" t="n">
-        <v>0.00223680000000000012</v>
+        <v>0.0016207</v>
       </c>
       <c r="D5" t="n">
-        <v>10.9800000000000004</v>
+        <v>1.85</v>
       </c>
       <c r="E5" t="n">
-        <v>26.9100000000000001</v>
+        <v>7.3</v>
       </c>
       <c r="F5" t="n">
-        <v>48.6899999999999977</v>
+        <v>14.61</v>
       </c>
       <c r="G5" t="n">
-        <v>77.1800000000000068</v>
+        <v>16.56</v>
       </c>
       <c r="H5" t="n">
-        <v>113.260000000000005</v>
+        <v>19.59</v>
       </c>
       <c r="I5" t="n">
-        <v>157.819999999999993</v>
+        <v>23.55</v>
       </c>
       <c r="J5" t="n">
-        <v>223.219999999999999</v>
+        <v>37.37</v>
       </c>
       <c r="K5" t="n">
-        <v>289.70999999999998</v>
+        <v>52.95</v>
       </c>
       <c r="L5" t="n">
-        <v>367.70999999999998</v>
+        <v>69.44</v>
       </c>
       <c r="M5" t="n">
-        <v>458.139999999999986</v>
+        <v>88.70999999999999</v>
       </c>
       <c r="N5" t="n">
-        <v>177.360000000000014</v>
-      </c>
-    </row>
-    <row r="6" spans="1:14">
+        <v>33.19</v>
+      </c>
+    </row>
+    <row r="6">
       <c r="A6" s="1" t="n">
         <v>4</v>
       </c>
@@ -650,43 +653,43 @@
         <v>9</v>
       </c>
       <c r="C6" t="n">
-        <v>0.0115280000000000005</v>
+        <v>0.0024063</v>
       </c>
       <c r="D6" t="n">
-        <v>13.5399999999999991</v>
+        <v>1.19</v>
       </c>
       <c r="E6" t="n">
-        <v>34.1499999999999986</v>
+        <v>5.35</v>
       </c>
       <c r="F6" t="n">
-        <v>63.240000000000002</v>
+        <v>10.54</v>
       </c>
       <c r="G6" t="n">
-        <v>102.180000000000007</v>
+        <v>9.74</v>
       </c>
       <c r="H6" t="n">
-        <v>152.379999999999995</v>
+        <v>9.26</v>
       </c>
       <c r="I6" t="n">
-        <v>215.219999999999999</v>
+        <v>8.99</v>
       </c>
       <c r="J6" t="n">
-        <v>306.569999999999993</v>
+        <v>16.54</v>
       </c>
       <c r="K6" t="n">
-        <v>402.279999999999973</v>
+        <v>24.52</v>
       </c>
       <c r="L6" t="n">
-        <v>515.440000000000055</v>
+        <v>32.27</v>
       </c>
       <c r="M6" t="n">
-        <v>647.490000000000009</v>
+        <v>41.31</v>
       </c>
       <c r="N6" t="n">
-        <v>245.25</v>
-      </c>
-    </row>
-    <row r="7" spans="1:14">
+        <v>15.97</v>
+      </c>
+    </row>
+    <row r="7">
       <c r="A7" s="1" t="n">
         <v>5</v>
       </c>
@@ -694,43 +697,43 @@
         <v>10</v>
       </c>
       <c r="C7" t="n">
-        <v>0.0240879999999999983</v>
+        <v>0.0024483</v>
       </c>
       <c r="D7" t="n">
-        <v>12.8000000000000007</v>
+        <v>1.32</v>
       </c>
       <c r="E7" t="n">
-        <v>31.6600000000000001</v>
+        <v>5.72</v>
       </c>
       <c r="F7" t="n">
-        <v>57.6599999999999966</v>
+        <v>11.29</v>
       </c>
       <c r="G7" t="n">
-        <v>91.9000000000000057</v>
+        <v>10.96</v>
       </c>
       <c r="H7" t="n">
-        <v>135.470000000000027</v>
+        <v>11.08</v>
       </c>
       <c r="I7" t="n">
-        <v>189.449999999999989</v>
+        <v>11.52</v>
       </c>
       <c r="J7" t="n">
-        <v>268.009999999999991</v>
+        <v>20.13</v>
       </c>
       <c r="K7" t="n">
-        <v>348.949999999999989</v>
+        <v>29.38</v>
       </c>
       <c r="L7" t="n">
-        <v>444.069999999999993</v>
+        <v>38.57</v>
       </c>
       <c r="M7" t="n">
-        <v>554.490000000000009</v>
+        <v>49.29</v>
       </c>
       <c r="N7" t="n">
-        <v>213.449999999999989</v>
-      </c>
-    </row>
-    <row r="8" spans="1:14">
+        <v>18.92</v>
+      </c>
+    </row>
+    <row r="8">
       <c r="A8" s="1" t="n">
         <v>6</v>
       </c>
@@ -738,43 +741,43 @@
         <v>11</v>
       </c>
       <c r="C8" t="n">
-        <v>0.0704720000000000013</v>
+        <v>0.00537</v>
       </c>
       <c r="D8" t="n">
-        <v>9.8100000000000005</v>
+        <v>0.48</v>
       </c>
       <c r="E8" t="n">
-        <v>23.6700000000000017</v>
+        <v>3.42</v>
       </c>
       <c r="F8" t="n">
-        <v>42.2299999999999969</v>
+        <v>6.7</v>
       </c>
       <c r="G8" t="n">
-        <v>66.1899999999999977</v>
+        <v>3.56</v>
       </c>
       <c r="H8" t="n">
-        <v>96.2000000000000028</v>
+        <v>0.19</v>
       </c>
       <c r="I8" t="n">
-        <v>132.949999999999989</v>
+        <v>3.49</v>
       </c>
       <c r="J8" t="n">
-        <v>187.319999999999993</v>
+        <v>0.92</v>
       </c>
       <c r="K8" t="n">
-        <v>241.490000000000009</v>
+        <v>1.11</v>
       </c>
       <c r="L8" t="n">
-        <v>304.730000000000018</v>
+        <v>2.11</v>
       </c>
       <c r="M8" t="n">
-        <v>377.740000000000009</v>
+        <v>3.38</v>
       </c>
       <c r="N8" t="n">
-        <v>148.22999999999999</v>
-      </c>
-    </row>
-    <row r="9" spans="1:14">
+        <v>2.54</v>
+      </c>
+    </row>
+    <row r="9">
       <c r="A9" s="1" t="n">
         <v>7</v>
       </c>
@@ -782,43 +785,43 @@
         <v>12</v>
       </c>
       <c r="C9" t="n">
-        <v>0.118710000000000004</v>
+        <v>0.0057857</v>
       </c>
       <c r="D9" t="n">
-        <v>5.45000000000000018</v>
+        <v>0.24</v>
       </c>
       <c r="E9" t="n">
-        <v>12.3000000000000007</v>
+        <v>2.75</v>
       </c>
       <c r="F9" t="n">
-        <v>20.7300000000000004</v>
+        <v>5.4</v>
       </c>
       <c r="G9" t="n">
-        <v>30.9400000000000013</v>
+        <v>1.48</v>
       </c>
       <c r="H9" t="n">
-        <v>43.1400000000000006</v>
+        <v>2.84</v>
       </c>
       <c r="I9" t="n">
-        <v>57.5</v>
+        <v>7.63</v>
       </c>
       <c r="J9" t="n">
-        <v>80.6500000000000057</v>
+        <v>6.68</v>
       </c>
       <c r="K9" t="n">
-        <v>100.650000000000006</v>
+        <v>6.59</v>
       </c>
       <c r="L9" t="n">
-        <v>123.510000000000005</v>
+        <v>7.76</v>
       </c>
       <c r="M9" t="n">
-        <v>149.430000000000007</v>
+        <v>9</v>
       </c>
       <c r="N9" t="n">
-        <v>62.4299999999999997</v>
-      </c>
-    </row>
-    <row r="10" spans="1:14">
+        <v>5.04</v>
+      </c>
+    </row>
+    <row r="10">
       <c r="A10" s="1" t="n">
         <v>8</v>
       </c>
@@ -826,43 +829,43 @@
         <v>13</v>
       </c>
       <c r="C10" t="n">
-        <v>0.13389000000000002</v>
+        <v>0.0061509</v>
       </c>
       <c r="D10" t="n">
-        <v>4.41000000000000014</v>
+        <v>0.03</v>
       </c>
       <c r="E10" t="n">
-        <v>9.59999999999999964</v>
+        <v>2.21</v>
       </c>
       <c r="F10" t="n">
-        <v>15.6500000000000004</v>
+        <v>4.36</v>
       </c>
       <c r="G10" t="n">
-        <v>22.6400000000000006</v>
+        <v>0.16</v>
       </c>
       <c r="H10" t="n">
-        <v>30.6700000000000017</v>
+        <v>5.2</v>
       </c>
       <c r="I10" t="n">
-        <v>39.8100000000000023</v>
+        <v>10.83</v>
       </c>
       <c r="J10" t="n">
-        <v>55.6899999999999977</v>
+        <v>11.1</v>
       </c>
       <c r="K10" t="n">
-        <v>67.75</v>
+        <v>12.45</v>
       </c>
       <c r="L10" t="n">
-        <v>81.230000000000004</v>
+        <v>15.24</v>
       </c>
       <c r="M10" t="n">
-        <v>96.2199999999999989</v>
+        <v>18.34</v>
       </c>
       <c r="N10" t="n">
-        <v>42.3699999999999974</v>
-      </c>
-    </row>
-    <row r="11" spans="1:14">
+        <v>7.99</v>
+      </c>
+    </row>
+    <row r="11">
       <c r="A11" s="1" t="n">
         <v>9</v>
       </c>
@@ -870,43 +873,43 @@
         <v>14</v>
       </c>
       <c r="C11" t="n">
-        <v>0.0974639999999999951</v>
+        <v>0.0061509</v>
       </c>
       <c r="D11" t="n">
-        <v>2.64999999999999991</v>
+        <v>0.03</v>
       </c>
       <c r="E11" t="n">
-        <v>5.29000000000000004</v>
+        <v>2.22</v>
       </c>
       <c r="F11" t="n">
-        <v>7.87999999999999989</v>
+        <v>4.37</v>
       </c>
       <c r="G11" t="n">
-        <v>10.4000000000000004</v>
+        <v>0.15</v>
       </c>
       <c r="H11" t="n">
-        <v>12.8100000000000005</v>
+        <v>5.19</v>
       </c>
       <c r="I11" t="n">
-        <v>15.0899999999999999</v>
+        <v>10.81</v>
       </c>
       <c r="J11" t="n">
-        <v>21.5300000000000011</v>
+        <v>11.07</v>
       </c>
       <c r="K11" t="n">
-        <v>23.5199999999999996</v>
+        <v>12.42</v>
       </c>
       <c r="L11" t="n">
-        <v>25.2800000000000011</v>
+        <v>15.2</v>
       </c>
       <c r="M11" t="n">
-        <v>26.7800000000000011</v>
+        <v>18.28</v>
       </c>
       <c r="N11" t="n">
-        <v>15.1199999999999992</v>
-      </c>
-    </row>
-    <row r="12" spans="1:14">
+        <v>7.97</v>
+      </c>
+    </row>
+    <row r="12">
       <c r="A12" s="1" t="n">
         <v>10</v>
       </c>
@@ -914,43 +917,43 @@
         <v>15</v>
       </c>
       <c r="C12" t="n">
-        <v>0.0974890000000000079</v>
+        <v>0.011126</v>
       </c>
       <c r="D12" t="n">
-        <v>2.62000000000000011</v>
+        <v>0.61</v>
       </c>
       <c r="E12" t="n">
-        <v>5.20999999999999996</v>
+        <v>3.65</v>
       </c>
       <c r="F12" t="n">
-        <v>7.74000000000000021</v>
+        <v>6.99</v>
       </c>
       <c r="G12" t="n">
-        <v>10.1699999999999999</v>
+        <v>3.82</v>
       </c>
       <c r="H12" t="n">
-        <v>12.4700000000000006</v>
+        <v>0.33</v>
       </c>
       <c r="I12" t="n">
-        <v>14.6099999999999994</v>
+        <v>3.56</v>
       </c>
       <c r="J12" t="n">
-        <v>20.8599999999999994</v>
+        <v>1.31</v>
       </c>
       <c r="K12" t="n">
-        <v>22.6499999999999986</v>
+        <v>0.25</v>
       </c>
       <c r="L12" t="n">
-        <v>24.1700000000000017</v>
+        <v>0.65</v>
       </c>
       <c r="M12" t="n">
-        <v>25.3999999999999986</v>
+        <v>1.15</v>
       </c>
       <c r="N12" t="n">
-        <v>14.5899999999999999</v>
-      </c>
-    </row>
-    <row r="13" spans="1:14">
+        <v>2.23</v>
+      </c>
+    </row>
+    <row r="13">
       <c r="A13" s="1" t="n">
         <v>11</v>
       </c>
@@ -958,43 +961,43 @@
         <v>16</v>
       </c>
       <c r="C13" t="n">
-        <v>0.142020000000000017</v>
+        <v>0.024096</v>
       </c>
       <c r="D13" t="n">
-        <v>3.62000000000000011</v>
+        <v>0.27</v>
       </c>
       <c r="E13" t="n">
-        <v>7.58000000000000007</v>
+        <v>2.67</v>
       </c>
       <c r="F13" t="n">
-        <v>11.9000000000000004</v>
+        <v>5.01</v>
       </c>
       <c r="G13" t="n">
-        <v>16.6000000000000014</v>
+        <v>0.57</v>
       </c>
       <c r="H13" t="n">
-        <v>21.6799999999999997</v>
+        <v>4.49</v>
       </c>
       <c r="I13" t="n">
-        <v>27.1700000000000017</v>
+        <v>10.23</v>
       </c>
       <c r="J13" t="n">
-        <v>37.990000000000002</v>
+        <v>10.68</v>
       </c>
       <c r="K13" t="n">
-        <v>44.5600000000000023</v>
+        <v>12.37</v>
       </c>
       <c r="L13" t="n">
-        <v>51.6000000000000014</v>
+        <v>15.64</v>
       </c>
       <c r="M13" t="n">
-        <v>59.1199999999999974</v>
+        <v>19.39</v>
       </c>
       <c r="N13" t="n">
-        <v>28.1799999999999997</v>
-      </c>
-    </row>
-    <row r="14" spans="1:14">
+        <v>8.130000000000001</v>
+      </c>
+    </row>
+    <row r="14">
       <c r="A14" s="1" t="n">
         <v>12</v>
       </c>
@@ -1002,43 +1005,43 @@
         <v>17</v>
       </c>
       <c r="C14" t="n">
-        <v>0.339760000000000018</v>
+        <v>0.015508</v>
       </c>
       <c r="D14" t="n">
-        <v>0.980000000000000071</v>
+        <v>0.96</v>
       </c>
       <c r="E14" t="n">
-        <v>1.25</v>
+        <v>0.4</v>
       </c>
       <c r="F14" t="n">
-        <v>0.689999999999999947</v>
+        <v>0.66</v>
       </c>
       <c r="G14" t="n">
-        <v>0.829999999999999893</v>
+        <v>8.039999999999999</v>
       </c>
       <c r="H14" t="n">
-        <v>3.41999999999999993</v>
+        <v>16.52</v>
       </c>
       <c r="I14" t="n">
-        <v>7.20999999999999996</v>
+        <v>26.12</v>
       </c>
       <c r="J14" t="n">
-        <v>9.08000000000000007</v>
+        <v>32.17</v>
       </c>
       <c r="K14" t="n">
-        <v>15.8800000000000008</v>
+        <v>40.35</v>
       </c>
       <c r="L14" t="n">
-        <v>24.2899999999999991</v>
+        <v>50.76</v>
       </c>
       <c r="M14" t="n">
-        <v>34.4399999999999977</v>
+        <v>62.57</v>
       </c>
       <c r="N14" t="n">
-        <v>9.8100000000000005</v>
-      </c>
-    </row>
-    <row r="15" spans="1:14">
+        <v>23.86</v>
+      </c>
+    </row>
+    <row r="15">
       <c r="A15" s="1" t="n">
         <v>13</v>
       </c>
@@ -1046,43 +1049,43 @@
         <v>18</v>
       </c>
       <c r="C15" t="n">
-        <v>0.268890000000000029</v>
+        <v>0.017391</v>
       </c>
       <c r="D15" t="n">
-        <v>3.97000000000000028</v>
+        <v>0.75</v>
       </c>
       <c r="E15" t="n">
-        <v>8.65000000000000036</v>
+        <v>0.13</v>
       </c>
       <c r="F15" t="n">
-        <v>14.1199999999999992</v>
+        <v>0.31</v>
       </c>
       <c r="G15" t="n">
-        <v>20.4699999999999989</v>
+        <v>6.56</v>
       </c>
       <c r="H15" t="n">
-        <v>27.7899999999999991</v>
+        <v>14.47</v>
       </c>
       <c r="I15" t="n">
-        <v>36.1499999999999986</v>
+        <v>23.42</v>
       </c>
       <c r="J15" t="n">
-        <v>51.0200000000000031</v>
+        <v>28.54</v>
       </c>
       <c r="K15" t="n">
-        <v>62.1400000000000006</v>
+        <v>35.63</v>
       </c>
       <c r="L15" t="n">
-        <v>74.5999999999999801</v>
+        <v>44.85</v>
       </c>
       <c r="M15" t="n">
-        <v>88.4899999999999807</v>
+        <v>55.33</v>
       </c>
       <c r="N15" t="n">
-        <v>38.740000000000002</v>
-      </c>
-    </row>
-    <row r="16" spans="1:14">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="16">
       <c r="A16" s="1" t="n">
         <v>14</v>
       </c>
@@ -1090,43 +1093,43 @@
         <v>19</v>
       </c>
       <c r="C16" t="n">
-        <v>0.278449999999999953</v>
+        <v>0.024235</v>
       </c>
       <c r="D16" t="n">
-        <v>4.76999999999999957</v>
+        <v>0.01</v>
       </c>
       <c r="E16" t="n">
-        <v>10.4499999999999993</v>
+        <v>1.93</v>
       </c>
       <c r="F16" t="n">
-        <v>17.149999999999995</v>
+        <v>3.58</v>
       </c>
       <c r="G16" t="n">
-        <v>24.9699999999999989</v>
+        <v>1.69</v>
       </c>
       <c r="H16" t="n">
-        <v>34.009999999999998</v>
+        <v>7.75</v>
       </c>
       <c r="I16" t="n">
-        <v>44.3599999999999994</v>
+        <v>14.65</v>
       </c>
       <c r="J16" t="n">
-        <v>61.8800000000000026</v>
+        <v>16.82</v>
       </c>
       <c r="K16" t="n">
-        <v>75.6500000000000057</v>
+        <v>20.54</v>
       </c>
       <c r="L16" t="n">
-        <v>91.0999999999999943</v>
+        <v>26.09</v>
       </c>
       <c r="M16" t="n">
-        <v>108.319999999999993</v>
+        <v>32.46</v>
       </c>
       <c r="N16" t="n">
-        <v>47.2700000000000031</v>
-      </c>
-    </row>
-    <row r="17" spans="1:14">
+        <v>12.55</v>
+      </c>
+    </row>
+    <row r="17">
       <c r="A17" s="1" t="n">
         <v>15</v>
       </c>
@@ -1134,43 +1137,43 @@
         <v>20</v>
       </c>
       <c r="C17" t="n">
-        <v>0.318940000000000001</v>
+        <v>0.024713</v>
       </c>
       <c r="D17" t="n">
-        <v>4.75999999999999979</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="E17" t="n">
-        <v>10.3900000000000006</v>
+        <v>2.12</v>
       </c>
       <c r="F17" t="n">
-        <v>16.9800000000000004</v>
+        <v>3.92</v>
       </c>
       <c r="G17" t="n">
-        <v>24.6099999999999994</v>
+        <v>1.17</v>
       </c>
       <c r="H17" t="n">
-        <v>33.3800000000000026</v>
+        <v>7.03</v>
       </c>
       <c r="I17" t="n">
-        <v>43.3699999999999974</v>
+        <v>13.71</v>
       </c>
       <c r="J17" t="n">
-        <v>60.3800000000000026</v>
+        <v>15.56</v>
       </c>
       <c r="K17" t="n">
-        <v>73.5600000000000023</v>
+        <v>18.9</v>
       </c>
       <c r="L17" t="n">
-        <v>88.2900000000000063</v>
+        <v>24.05</v>
       </c>
       <c r="M17" t="n">
-        <v>104.659999999999997</v>
+        <v>29.97</v>
       </c>
       <c r="N17" t="n">
-        <v>46.0399999999999991</v>
-      </c>
-    </row>
-    <row r="18" spans="1:14">
+        <v>11.65</v>
+      </c>
+    </row>
+    <row r="18">
       <c r="A18" s="1" t="n">
         <v>16</v>
       </c>
@@ -1178,43 +1181,43 @@
         <v>21</v>
       </c>
       <c r="C18" t="n">
-        <v>0.349129999999999985</v>
+        <v>0.021901</v>
       </c>
       <c r="D18" t="n">
-        <v>2.12000000000000011</v>
+        <v>0.14</v>
       </c>
       <c r="E18" t="n">
-        <v>4.16000000000000014</v>
+        <v>2.32</v>
       </c>
       <c r="F18" t="n">
-        <v>6.12000000000000011</v>
+        <v>4.3</v>
       </c>
       <c r="G18" t="n">
-        <v>7.96999999999999975</v>
+        <v>0.57</v>
       </c>
       <c r="H18" t="n">
-        <v>9.73000000000000043</v>
+        <v>6.16</v>
       </c>
       <c r="I18" t="n">
-        <v>11.3699999999999992</v>
+        <v>12.55</v>
       </c>
       <c r="J18" t="n">
-        <v>17.0399999999999991</v>
+        <v>13.96</v>
       </c>
       <c r="K18" t="n">
-        <v>18.4699999999999989</v>
+        <v>16.79</v>
       </c>
       <c r="L18" t="n">
-        <v>19.75</v>
+        <v>21.37</v>
       </c>
       <c r="M18" t="n">
-        <v>20.870000000000001</v>
+        <v>26.64</v>
       </c>
       <c r="N18" t="n">
-        <v>11.7599999999999998</v>
-      </c>
-    </row>
-    <row r="19" spans="1:14">
+        <v>10.48</v>
+      </c>
+    </row>
+    <row r="19">
       <c r="A19" s="1" t="n">
         <v>17</v>
       </c>
@@ -1222,43 +1225,43 @@
         <v>22</v>
       </c>
       <c r="C19" t="n">
-        <v>0.363020000000000032</v>
+        <v>0.026602</v>
       </c>
       <c r="D19" t="n">
-        <v>1.82000000000000011</v>
+        <v>0.2</v>
       </c>
       <c r="E19" t="n">
-        <v>3.45999999999999996</v>
+        <v>2.45</v>
       </c>
       <c r="F19" t="n">
-        <v>4.90000000000000036</v>
+        <v>4.51</v>
       </c>
       <c r="G19" t="n">
-        <v>6.09999999999999964</v>
+        <v>0.29</v>
       </c>
       <c r="H19" t="n">
-        <v>7.05999999999999961</v>
+        <v>5.82</v>
       </c>
       <c r="I19" t="n">
-        <v>7.75</v>
+        <v>12.13</v>
       </c>
       <c r="J19" t="n">
-        <v>12.1400000000000006</v>
+        <v>13.45</v>
       </c>
       <c r="K19" t="n">
-        <v>12.2300000000000004</v>
+        <v>16.18</v>
       </c>
       <c r="L19" t="n">
-        <v>11.9700000000000006</v>
+        <v>20.68</v>
       </c>
       <c r="M19" t="n">
-        <v>11.3499999999999996</v>
+        <v>25.85</v>
       </c>
       <c r="N19" t="n">
-        <v>7.87999999999999989</v>
-      </c>
-    </row>
-    <row r="20" spans="1:14">
+        <v>10.16</v>
+      </c>
+    </row>
+    <row r="20">
       <c r="A20" s="1" t="n">
         <v>18</v>
       </c>
@@ -1266,43 +1269,43 @@
         <v>23</v>
       </c>
       <c r="C20" t="n">
-        <v>0.463539999999999974</v>
+        <v>0.032967</v>
       </c>
       <c r="D20" t="n">
-        <v>2.08000000000000007</v>
+        <v>0.41</v>
       </c>
       <c r="E20" t="n">
-        <v>4.09999999999999964</v>
+        <v>2.96</v>
       </c>
       <c r="F20" t="n">
-        <v>6.03000000000000025</v>
+        <v>5.43</v>
       </c>
       <c r="G20" t="n">
-        <v>7.87000000000000011</v>
+        <v>1.08</v>
       </c>
       <c r="H20" t="n">
-        <v>9.59999999999999964</v>
+        <v>3.94</v>
       </c>
       <c r="I20" t="n">
-        <v>11.2300000000000004</v>
+        <v>9.69</v>
       </c>
       <c r="J20" t="n">
-        <v>16.899999999999995</v>
+        <v>10.2</v>
       </c>
       <c r="K20" t="n">
-        <v>18.3299999999999983</v>
+        <v>12</v>
       </c>
       <c r="L20" t="n">
-        <v>19.620000000000001</v>
+        <v>15.5</v>
       </c>
       <c r="M20" t="n">
-        <v>20.75</v>
+        <v>19.55</v>
       </c>
       <c r="N20" t="n">
-        <v>11.6500000000000004</v>
-      </c>
-    </row>
-    <row r="21" spans="1:14">
+        <v>8.07</v>
+      </c>
+    </row>
+    <row r="21">
       <c r="A21" s="1" t="n">
         <v>19</v>
       </c>
@@ -1310,43 +1313,43 @@
         <v>24</v>
       </c>
       <c r="C21" t="n">
-        <v>0.438490000000000002</v>
+        <v>0.035711</v>
       </c>
       <c r="D21" t="n">
-        <v>3</v>
+        <v>0.73</v>
       </c>
       <c r="E21" t="n">
-        <v>6.32000000000000028</v>
+        <v>3.73</v>
       </c>
       <c r="F21" t="n">
-        <v>9.97000000000000064</v>
+        <v>6.83</v>
       </c>
       <c r="G21" t="n">
-        <v>14</v>
+        <v>3.17</v>
       </c>
       <c r="H21" t="n">
-        <v>18.4400000000000013</v>
+        <v>1.07</v>
       </c>
       <c r="I21" t="n">
-        <v>23.3200000000000003</v>
+        <v>5.96</v>
       </c>
       <c r="J21" t="n">
-        <v>33.4200000000000017</v>
+        <v>5.22</v>
       </c>
       <c r="K21" t="n">
-        <v>39.5</v>
+        <v>5.62</v>
       </c>
       <c r="L21" t="n">
-        <v>46.1400000000000006</v>
+        <v>7.58</v>
       </c>
       <c r="M21" t="n">
-        <v>53.3800000000000026</v>
+        <v>9.92</v>
       </c>
       <c r="N21" t="n">
-        <v>24.75</v>
-      </c>
-    </row>
-    <row r="22" spans="1:14">
+        <v>4.98</v>
+      </c>
+    </row>
+    <row r="22">
       <c r="A22" s="1" t="n">
         <v>20</v>
       </c>
@@ -1354,43 +1357,43 @@
         <v>25</v>
       </c>
       <c r="C22" t="n">
-        <v>0.456430000000000025</v>
+        <v>0.035732</v>
       </c>
       <c r="D22" t="n">
-        <v>3.43000000000000016</v>
+        <v>0.72</v>
       </c>
       <c r="E22" t="n">
-        <v>7.26999999999999869</v>
+        <v>3.71</v>
       </c>
       <c r="F22" t="n">
-        <v>11.5600000000000005</v>
+        <v>6.8</v>
       </c>
       <c r="G22" t="n">
-        <v>16.3299999999999983</v>
+        <v>3.12</v>
       </c>
       <c r="H22" t="n">
-        <v>21.6400000000000006</v>
+        <v>1.14</v>
       </c>
       <c r="I22" t="n">
-        <v>27.5100000000000016</v>
+        <v>6.05</v>
       </c>
       <c r="J22" t="n">
-        <v>38.9299999999999997</v>
+        <v>5.34</v>
       </c>
       <c r="K22" t="n">
-        <v>46.3100000000000023</v>
+        <v>5.77</v>
       </c>
       <c r="L22" t="n">
-        <v>54.4099999999999966</v>
+        <v>7.77</v>
       </c>
       <c r="M22" t="n">
-        <v>63.259999999999998</v>
+        <v>10.15</v>
       </c>
       <c r="N22" t="n">
-        <v>29.0599999999999987</v>
-      </c>
-    </row>
-    <row r="23" spans="1:14">
+        <v>5.06</v>
+      </c>
+    </row>
+    <row r="23">
       <c r="A23" s="1" t="n">
         <v>21</v>
       </c>
@@ -1398,43 +1401,43 @@
         <v>26</v>
       </c>
       <c r="C23" t="n">
-        <v>0.519700000000000095</v>
+        <v>0.036944</v>
       </c>
       <c r="D23" t="n">
-        <v>2.91000000000000014</v>
+        <v>0.66</v>
       </c>
       <c r="E23" t="n">
-        <v>6.05999999999999961</v>
+        <v>3.57</v>
       </c>
       <c r="F23" t="n">
-        <v>9.47000000000000064</v>
+        <v>6.55</v>
       </c>
       <c r="G23" t="n">
-        <v>13.1600000000000001</v>
+        <v>2.75</v>
       </c>
       <c r="H23" t="n">
-        <v>17.1400000000000006</v>
+        <v>1.63</v>
       </c>
       <c r="I23" t="n">
-        <v>21.4499999999999993</v>
+        <v>6.68</v>
       </c>
       <c r="J23" t="n">
-        <v>30.7600000000000016</v>
+        <v>6.17</v>
       </c>
       <c r="K23" t="n">
-        <v>35.9699999999999989</v>
+        <v>6.82</v>
       </c>
       <c r="L23" t="n">
-        <v>41.5900000000000034</v>
+        <v>9.06</v>
       </c>
       <c r="M23" t="n">
-        <v>47.6300000000000026</v>
+        <v>11.71</v>
       </c>
       <c r="N23" t="n">
-        <v>22.620000000000001</v>
-      </c>
-    </row>
-    <row r="24" spans="1:14">
+        <v>5.56</v>
+      </c>
+    </row>
+    <row r="24">
       <c r="A24" s="1" t="n">
         <v>22</v>
       </c>
@@ -1442,43 +1445,43 @@
         <v>27</v>
       </c>
       <c r="C24" t="n">
-        <v>0.578669999999999973</v>
+        <v>0.04407</v>
       </c>
       <c r="D24" t="n">
-        <v>2.14000000000000012</v>
+        <v>0.68</v>
       </c>
       <c r="E24" t="n">
-        <v>4.26999999999999957</v>
+        <v>3.6</v>
       </c>
       <c r="F24" t="n">
-        <v>6.38999999999999968</v>
+        <v>6.59</v>
       </c>
       <c r="G24" t="n">
-        <v>8.5</v>
+        <v>2.8</v>
       </c>
       <c r="H24" t="n">
-        <v>10.5999999999999996</v>
+        <v>1.58</v>
       </c>
       <c r="I24" t="n">
-        <v>12.6999999999999993</v>
+        <v>6.65</v>
       </c>
       <c r="J24" t="n">
-        <v>19.0199999999999996</v>
+        <v>6.15</v>
       </c>
       <c r="K24" t="n">
-        <v>21.1799999999999997</v>
+        <v>6.82</v>
       </c>
       <c r="L24" t="n">
-        <v>23.3399999999999999</v>
+        <v>9.09</v>
       </c>
       <c r="M24" t="n">
-        <v>25.5</v>
+        <v>11.77</v>
       </c>
       <c r="N24" t="n">
-        <v>13.3599999999999994</v>
-      </c>
-    </row>
-    <row r="25" spans="1:14">
+        <v>5.57</v>
+      </c>
+    </row>
+    <row r="25">
       <c r="A25" s="1" t="n">
         <v>23</v>
       </c>
@@ -1486,43 +1489,43 @@
         <v>28</v>
       </c>
       <c r="C25" t="n">
-        <v>0.518120000000000047</v>
+        <v>0.04407</v>
       </c>
       <c r="D25" t="n">
-        <v>2</v>
+        <v>0.67</v>
       </c>
       <c r="E25" t="n">
-        <v>3.91999999999999993</v>
+        <v>3.6</v>
       </c>
       <c r="F25" t="n">
-        <v>5.75999999999999979</v>
+        <v>6.59</v>
       </c>
       <c r="G25" t="n">
-        <v>7.50999999999999979</v>
+        <v>2.8</v>
       </c>
       <c r="H25" t="n">
-        <v>9.16999999999999993</v>
+        <v>1.59</v>
       </c>
       <c r="I25" t="n">
-        <v>10.7300000000000004</v>
+        <v>6.65</v>
       </c>
       <c r="J25" t="n">
-        <v>16.3200000000000003</v>
+        <v>6.16</v>
       </c>
       <c r="K25" t="n">
-        <v>17.7100000000000009</v>
+        <v>6.83</v>
       </c>
       <c r="L25" t="n">
-        <v>18.9800000000000004</v>
+        <v>9.1</v>
       </c>
       <c r="M25" t="n">
-        <v>20.129999999999999</v>
+        <v>11.79</v>
       </c>
       <c r="N25" t="n">
-        <v>11.2200000000000006</v>
-      </c>
-    </row>
-    <row r="26" spans="1:14">
+        <v>5.58</v>
+      </c>
+    </row>
+    <row r="26">
       <c r="A26" s="1" t="n">
         <v>24</v>
       </c>
@@ -1530,43 +1533,43 @@
         <v>29</v>
       </c>
       <c r="C26" t="n">
-        <v>0.541500000000000004</v>
+        <v>0.051853</v>
       </c>
       <c r="D26" t="n">
-        <v>1.82000000000000011</v>
+        <v>0.25</v>
       </c>
       <c r="E26" t="n">
-        <v>3.50999999999999979</v>
+        <v>2.61</v>
       </c>
       <c r="F26" t="n">
-        <v>5.05999999999999961</v>
+        <v>4.86</v>
       </c>
       <c r="G26" t="n">
-        <v>6.46999999999999975</v>
+        <v>0.31</v>
       </c>
       <c r="H26" t="n">
-        <v>7.71999999999999975</v>
+        <v>4.9</v>
       </c>
       <c r="I26" t="n">
-        <v>8.80000000000000071</v>
+        <v>10.85</v>
       </c>
       <c r="J26" t="n">
-        <v>13.7599999999999998</v>
+        <v>11.63</v>
       </c>
       <c r="K26" t="n">
-        <v>14.5</v>
+        <v>13.73</v>
       </c>
       <c r="L26" t="n">
-        <v>15.0500000000000007</v>
+        <v>17.49</v>
       </c>
       <c r="M26" t="n">
-        <v>15.3699999999999992</v>
+        <v>21.84</v>
       </c>
       <c r="N26" t="n">
-        <v>9.21000000000000085</v>
-      </c>
-    </row>
-    <row r="27" spans="1:14">
+        <v>8.85</v>
+      </c>
+    </row>
+    <row r="27">
       <c r="A27" s="1" t="n">
         <v>25</v>
       </c>
@@ -1574,81 +1577,43 @@
         <v>30</v>
       </c>
       <c r="C27" t="n">
-        <v>0.555349999999999966</v>
+        <v>0.053035</v>
       </c>
       <c r="D27" t="n">
-        <v>1.95</v>
+        <v>0.2</v>
       </c>
       <c r="E27" t="n">
-        <v>3.79999999999999982</v>
+        <v>2.51</v>
       </c>
       <c r="F27" t="n">
-        <v>5.55999999999999961</v>
+        <v>4.69</v>
       </c>
       <c r="G27" t="n">
-        <v>7.20999999999999996</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="H27" t="n">
-        <v>8.75</v>
+        <v>5.23</v>
       </c>
       <c r="I27" t="n">
-        <v>10.1600000000000001</v>
+        <v>11.27</v>
       </c>
       <c r="J27" t="n">
-        <v>15.5600000000000005</v>
+        <v>12.17</v>
       </c>
       <c r="K27" t="n">
-        <v>16.7600000000000016</v>
+        <v>14.41</v>
       </c>
       <c r="L27" t="n">
-        <v>17.8099999999999952</v>
+        <v>18.33</v>
       </c>
       <c r="M27" t="n">
-        <v>18.7100000000000009</v>
+        <v>22.83</v>
       </c>
       <c r="N27" t="n">
-        <v>10.6300000000000008</v>
+        <v>9.17</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="D2:M27">
-    <cfRule type="colorScale" priority="1">
-      <colorScale>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="20"/>
-        <cfvo type="num" val="100"/>
-        <color rgb="FF3E76C1"/>
-        <color rgb="FFF36F0C"/>
-        <color rgb="FFFF0000"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <printOptions>
-    <extLst>
-      <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1699203626" printRowHead="0" printColHead="0" printHeadLine="0" printFootLine="0" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
-      </ext>
-    </extLst>
-  </printOptions>
-  <pageMargins left="0.750000" right="0.750000" top="1.000000" bottom="1.000000" header="0.500000" footer="0.500000"/>
-  <pageSetup paperSize="1" fitToWidth="0" fitToHeight="1" pageOrder="overThenDown"/>
-  <headerFooter>
-    <extLst>
-      <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1699203626" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1699203626" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
-        <pm:paperBin xmlns:pm="smNativeData" id="1699203626" Id="0" type="0" value="0"/>
-        <pm:paperBin xmlns:pm="smNativeData" id="1699203626" Id="1" type="0" value="0"/>
-      </ext>
-    </extLst>
-  </headerFooter>
-  <extLst>
-    <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1699203626" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
-        <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
-        <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
-      </pm:sheetPrefs>
-    </ext>
-  </extLst>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Updated on 11-06-2023 at 12:57
</commit_message>
<xml_diff>
--- a/output/accuracy_cubic.xlsx
+++ b/output/accuracy_cubic.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N14"/>
+  <dimension ref="A1:N27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -474,43 +474,43 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>18</v>
+        <v>5</v>
       </c>
       <c r="C2" t="n">
-        <v>0.009298799999999999</v>
+        <v>2.1806e-05</v>
       </c>
       <c r="D2" t="n">
-        <v>29.58</v>
+        <v>0.61</v>
       </c>
       <c r="E2" t="n">
-        <v>25.8</v>
+        <v>2.14</v>
       </c>
       <c r="F2" t="n">
-        <v>30.77</v>
+        <v>6.13</v>
       </c>
       <c r="G2" t="n">
-        <v>8.07</v>
+        <v>14.22</v>
       </c>
       <c r="H2" t="n">
-        <v>8.08</v>
+        <v>22.54</v>
       </c>
       <c r="I2" t="n">
-        <v>4.8</v>
+        <v>35.19</v>
       </c>
       <c r="J2" t="n">
-        <v>6.32</v>
+        <v>51.66</v>
       </c>
       <c r="K2" t="n">
-        <v>1.73</v>
+        <v>71.62</v>
       </c>
       <c r="L2" t="n">
-        <v>0.21</v>
+        <v>95.90000000000001</v>
       </c>
       <c r="M2" t="n">
-        <v>1.22</v>
+        <v>125.64</v>
       </c>
       <c r="N2" t="n">
-        <v>11.66</v>
+        <v>42.57</v>
       </c>
     </row>
     <row r="3">
@@ -518,43 +518,43 @@
         <v>1</v>
       </c>
       <c r="B3" t="n">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="C3" t="n">
-        <v>0.0114</v>
+        <v>0.00030075</v>
       </c>
       <c r="D3" t="n">
-        <v>77.20999999999999</v>
+        <v>2</v>
       </c>
       <c r="E3" t="n">
-        <v>132.67</v>
+        <v>6.35</v>
       </c>
       <c r="F3" t="n">
-        <v>218.66</v>
+        <v>12.46</v>
       </c>
       <c r="G3" t="n">
-        <v>238.18</v>
+        <v>18.93</v>
       </c>
       <c r="H3" t="n">
-        <v>325.25</v>
+        <v>31.9</v>
       </c>
       <c r="I3" t="n">
-        <v>410.4</v>
+        <v>46.57</v>
       </c>
       <c r="J3" t="n">
-        <v>534.04</v>
+        <v>64</v>
       </c>
       <c r="K3" t="n">
-        <v>613.22</v>
+        <v>86.5</v>
       </c>
       <c r="L3" t="n">
-        <v>779.5599999999999</v>
+        <v>116.46</v>
       </c>
       <c r="M3" t="n">
-        <v>985.8200000000001</v>
+        <v>150.16</v>
       </c>
       <c r="N3" t="n">
-        <v>431.5</v>
+        <v>53.53</v>
       </c>
     </row>
     <row r="4">
@@ -562,43 +562,43 @@
         <v>2</v>
       </c>
       <c r="B4" t="n">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="C4" t="n">
-        <v>0.01705</v>
+        <v>4.9872e-06</v>
       </c>
       <c r="D4" t="n">
-        <v>93.89</v>
+        <v>0.74</v>
       </c>
       <c r="E4" t="n">
-        <v>168.64</v>
+        <v>1.96</v>
       </c>
       <c r="F4" t="n">
-        <v>280.11</v>
+        <v>4.78</v>
       </c>
       <c r="G4" t="n">
-        <v>311.83</v>
+        <v>10.52</v>
       </c>
       <c r="H4" t="n">
-        <v>425.07</v>
+        <v>14.82</v>
       </c>
       <c r="I4" t="n">
-        <v>536.37</v>
+        <v>21.65</v>
       </c>
       <c r="J4" t="n">
-        <v>696.1900000000001</v>
+        <v>30.24</v>
       </c>
       <c r="K4" t="n">
-        <v>800.5</v>
+        <v>39.77</v>
       </c>
       <c r="L4" t="n">
-        <v>1015.31</v>
+        <v>50.21</v>
       </c>
       <c r="M4" t="n">
-        <v>1281.66</v>
+        <v>63.06</v>
       </c>
       <c r="N4" t="n">
-        <v>560.96</v>
+        <v>23.77</v>
       </c>
     </row>
     <row r="5">
@@ -606,43 +606,43 @@
         <v>3</v>
       </c>
       <c r="B5" t="n">
-        <v>21</v>
+        <v>8</v>
       </c>
       <c r="C5" t="n">
-        <v>0.0063699</v>
+        <v>2.0719e-05</v>
       </c>
       <c r="D5" t="n">
-        <v>75.65000000000001</v>
+        <v>0.55</v>
       </c>
       <c r="E5" t="n">
-        <v>131.06</v>
+        <v>1.97</v>
       </c>
       <c r="F5" t="n">
-        <v>218.23</v>
+        <v>5.76</v>
       </c>
       <c r="G5" t="n">
-        <v>239.89</v>
+        <v>13.56</v>
       </c>
       <c r="H5" t="n">
-        <v>330.02</v>
+        <v>21.46</v>
       </c>
       <c r="I5" t="n">
-        <v>419</v>
+        <v>33.6</v>
       </c>
       <c r="J5" t="n">
-        <v>547.91</v>
+        <v>49.41</v>
       </c>
       <c r="K5" t="n">
-        <v>632.01</v>
+        <v>68.56999999999999</v>
       </c>
       <c r="L5" t="n">
-        <v>806.24</v>
+        <v>91.83</v>
       </c>
       <c r="M5" t="n">
-        <v>1022.61</v>
+        <v>120.37</v>
       </c>
       <c r="N5" t="n">
-        <v>442.26</v>
+        <v>40.71</v>
       </c>
     </row>
     <row r="6">
@@ -650,43 +650,43 @@
         <v>4</v>
       </c>
       <c r="B6" t="n">
-        <v>22</v>
+        <v>9</v>
       </c>
       <c r="C6" t="n">
-        <v>0.010574</v>
+        <v>0.00068176</v>
       </c>
       <c r="D6" t="n">
-        <v>68.37</v>
+        <v>1.04</v>
       </c>
       <c r="E6" t="n">
-        <v>115.59</v>
+        <v>2.36</v>
       </c>
       <c r="F6" t="n">
-        <v>192.12</v>
+        <v>4.95</v>
       </c>
       <c r="G6" t="n">
-        <v>208.92</v>
+        <v>10.05</v>
       </c>
       <c r="H6" t="n">
-        <v>288.4</v>
+        <v>13.16</v>
       </c>
       <c r="I6" t="n">
-        <v>366.87</v>
+        <v>18.19</v>
       </c>
       <c r="J6" t="n">
-        <v>481.25</v>
+        <v>24.32</v>
       </c>
       <c r="K6" t="n">
-        <v>555.4400000000001</v>
+        <v>30.59</v>
       </c>
       <c r="L6" t="n">
-        <v>710.35</v>
+        <v>36.71</v>
       </c>
       <c r="M6" t="n">
-        <v>902.8099999999999</v>
+        <v>44.28</v>
       </c>
       <c r="N6" t="n">
-        <v>389.01</v>
+        <v>18.57</v>
       </c>
     </row>
     <row r="7">
@@ -694,43 +694,43 @@
         <v>5</v>
       </c>
       <c r="B7" t="n">
-        <v>23</v>
+        <v>10</v>
       </c>
       <c r="C7" t="n">
-        <v>0.016136</v>
+        <v>0.00069472</v>
       </c>
       <c r="D7" t="n">
-        <v>69.56999999999999</v>
+        <v>0.87</v>
       </c>
       <c r="E7" t="n">
-        <v>116.51</v>
+        <v>1.88</v>
       </c>
       <c r="F7" t="n">
-        <v>191.47</v>
+        <v>3.98</v>
       </c>
       <c r="G7" t="n">
-        <v>206.01</v>
+        <v>8.43</v>
       </c>
       <c r="H7" t="n">
-        <v>282.11</v>
+        <v>10.65</v>
       </c>
       <c r="I7" t="n">
-        <v>356.46</v>
+        <v>14.57</v>
       </c>
       <c r="J7" t="n">
-        <v>465.16</v>
+        <v>19.38</v>
       </c>
       <c r="K7" t="n">
-        <v>534.21</v>
+        <v>24.03</v>
       </c>
       <c r="L7" t="n">
-        <v>680.72</v>
+        <v>28.12</v>
       </c>
       <c r="M7" t="n">
-        <v>862.47</v>
+        <v>33.36</v>
       </c>
       <c r="N7" t="n">
-        <v>376.47</v>
+        <v>14.53</v>
       </c>
     </row>
     <row r="8">
@@ -738,43 +738,43 @@
         <v>6</v>
       </c>
       <c r="B8" t="n">
-        <v>24</v>
+        <v>11</v>
       </c>
       <c r="C8" t="n">
-        <v>0.026899</v>
+        <v>0.00042211</v>
       </c>
       <c r="D8" t="n">
-        <v>63.84</v>
+        <v>0.4</v>
       </c>
       <c r="E8" t="n">
-        <v>103.75</v>
+        <v>0.49</v>
       </c>
       <c r="F8" t="n">
-        <v>169.16</v>
+        <v>1.2</v>
       </c>
       <c r="G8" t="n">
-        <v>178.79</v>
+        <v>3.78</v>
       </c>
       <c r="H8" t="n">
-        <v>244.7</v>
+        <v>3.39</v>
       </c>
       <c r="I8" t="n">
-        <v>308.72</v>
+        <v>4.13</v>
       </c>
       <c r="J8" t="n">
-        <v>403.15</v>
+        <v>5.14</v>
       </c>
       <c r="K8" t="n">
-        <v>462.05</v>
+        <v>5.15</v>
       </c>
       <c r="L8" t="n">
-        <v>589.34</v>
+        <v>3.42</v>
       </c>
       <c r="M8" t="n">
-        <v>747.1900000000001</v>
+        <v>2.02</v>
       </c>
       <c r="N8" t="n">
-        <v>327.07</v>
+        <v>2.91</v>
       </c>
     </row>
     <row r="9">
@@ -782,43 +782,43 @@
         <v>7</v>
       </c>
       <c r="B9" t="n">
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="C9" t="n">
-        <v>0.042463</v>
+        <v>0.00065234</v>
       </c>
       <c r="D9" t="n">
-        <v>49.06</v>
+        <v>0.67</v>
       </c>
       <c r="E9" t="n">
-        <v>73.53</v>
+        <v>1.23</v>
       </c>
       <c r="F9" t="n">
-        <v>119.76</v>
+        <v>2.6</v>
       </c>
       <c r="G9" t="n">
-        <v>121.75</v>
+        <v>6.03</v>
       </c>
       <c r="H9" t="n">
-        <v>169.83</v>
+        <v>6.81</v>
       </c>
       <c r="I9" t="n">
-        <v>216.84</v>
+        <v>8.949999999999999</v>
       </c>
       <c r="J9" t="n">
-        <v>287.74</v>
+        <v>11.59</v>
       </c>
       <c r="K9" t="n">
-        <v>331.61</v>
+        <v>13.59</v>
       </c>
       <c r="L9" t="n">
-        <v>428.3</v>
+        <v>14.33</v>
       </c>
       <c r="M9" t="n">
-        <v>548.6</v>
+        <v>15.73</v>
       </c>
       <c r="N9" t="n">
-        <v>234.7</v>
+        <v>8.15</v>
       </c>
     </row>
     <row r="10">
@@ -826,43 +826,43 @@
         <v>8</v>
       </c>
       <c r="B10" t="n">
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="C10" t="n">
-        <v>0.050982</v>
+        <v>0.0013741</v>
       </c>
       <c r="D10" t="n">
-        <v>30.05</v>
+        <v>1</v>
       </c>
       <c r="E10" t="n">
-        <v>29.46</v>
+        <v>2.17</v>
       </c>
       <c r="F10" t="n">
-        <v>40.79</v>
+        <v>4.49</v>
       </c>
       <c r="G10" t="n">
-        <v>23.95</v>
+        <v>9.18</v>
       </c>
       <c r="H10" t="n">
-        <v>34.13</v>
+        <v>11.69</v>
       </c>
       <c r="I10" t="n">
-        <v>42.67</v>
+        <v>15.95</v>
       </c>
       <c r="J10" t="n">
-        <v>60.76</v>
+        <v>21.12</v>
       </c>
       <c r="K10" t="n">
-        <v>67.03</v>
+        <v>26.18</v>
       </c>
       <c r="L10" t="n">
-        <v>92.98999999999999</v>
+        <v>30.76</v>
       </c>
       <c r="M10" t="n">
-        <v>125.72</v>
+        <v>36.54</v>
       </c>
       <c r="N10" t="n">
-        <v>54.76</v>
+        <v>15.91</v>
       </c>
     </row>
     <row r="11">
@@ -870,43 +870,43 @@
         <v>9</v>
       </c>
       <c r="B11" t="n">
-        <v>27</v>
+        <v>14</v>
       </c>
       <c r="C11" t="n">
-        <v>0.052594</v>
+        <v>0.00033859</v>
       </c>
       <c r="D11" t="n">
-        <v>26.85</v>
+        <v>1.07</v>
       </c>
       <c r="E11" t="n">
-        <v>22.86</v>
+        <v>2.18</v>
       </c>
       <c r="F11" t="n">
-        <v>29.93</v>
+        <v>4.28</v>
       </c>
       <c r="G11" t="n">
-        <v>11.34</v>
+        <v>8.57</v>
       </c>
       <c r="H11" t="n">
-        <v>17.51</v>
+        <v>10.46</v>
       </c>
       <c r="I11" t="n">
-        <v>22.2</v>
+        <v>13.88</v>
       </c>
       <c r="J11" t="n">
-        <v>34.97</v>
+        <v>17.99</v>
       </c>
       <c r="K11" t="n">
-        <v>37.81</v>
+        <v>21.7</v>
       </c>
       <c r="L11" t="n">
-        <v>56.84</v>
+        <v>24.56</v>
       </c>
       <c r="M11" t="n">
-        <v>81.06999999999999</v>
+        <v>28.3</v>
       </c>
       <c r="N11" t="n">
-        <v>34.14</v>
+        <v>13.3</v>
       </c>
     </row>
     <row r="12">
@@ -914,43 +914,43 @@
         <v>10</v>
       </c>
       <c r="B12" t="n">
-        <v>28</v>
+        <v>15</v>
       </c>
       <c r="C12" t="n">
-        <v>0.054507</v>
+        <v>0.00065228</v>
       </c>
       <c r="D12" t="n">
-        <v>34.96</v>
+        <v>0.67</v>
       </c>
       <c r="E12" t="n">
-        <v>44.32</v>
+        <v>1.22</v>
       </c>
       <c r="F12" t="n">
-        <v>71.45999999999999</v>
+        <v>2.59</v>
       </c>
       <c r="G12" t="n">
-        <v>65.43000000000001</v>
+        <v>6.02</v>
       </c>
       <c r="H12" t="n">
-        <v>95.22</v>
+        <v>6.78</v>
       </c>
       <c r="I12" t="n">
-        <v>124.53</v>
+        <v>8.91</v>
       </c>
       <c r="J12" t="n">
-        <v>170.94</v>
+        <v>11.55</v>
       </c>
       <c r="K12" t="n">
-        <v>198.72</v>
+        <v>13.53</v>
       </c>
       <c r="L12" t="n">
-        <v>263.23</v>
+        <v>14.26</v>
       </c>
       <c r="M12" t="n">
-        <v>343.9</v>
+        <v>15.64</v>
       </c>
       <c r="N12" t="n">
-        <v>141.27</v>
+        <v>8.119999999999999</v>
       </c>
     </row>
     <row r="13">
@@ -958,43 +958,43 @@
         <v>11</v>
       </c>
       <c r="B13" t="n">
-        <v>29</v>
+        <v>16</v>
       </c>
       <c r="C13" t="n">
-        <v>0.00039979</v>
+        <v>0.0016352</v>
       </c>
       <c r="D13" t="n">
-        <v>20.79</v>
+        <v>1.46</v>
       </c>
       <c r="E13" t="n">
-        <v>9.77</v>
+        <v>3.28</v>
       </c>
       <c r="F13" t="n">
-        <v>7.6</v>
+        <v>6.42</v>
       </c>
       <c r="G13" t="n">
-        <v>15.31</v>
+        <v>12.09</v>
       </c>
       <c r="H13" t="n">
-        <v>18.43</v>
+        <v>15.87</v>
       </c>
       <c r="I13" t="n">
-        <v>22.86</v>
+        <v>21.57</v>
       </c>
       <c r="J13" t="n">
-        <v>22.65</v>
+        <v>28.38</v>
       </c>
       <c r="K13" t="n">
-        <v>28.3</v>
+        <v>35.37</v>
       </c>
       <c r="L13" t="n">
-        <v>25.81</v>
+        <v>42.32</v>
       </c>
       <c r="M13" t="n">
-        <v>21.96</v>
+        <v>50.72</v>
       </c>
       <c r="N13" t="n">
-        <v>19.35</v>
+        <v>21.75</v>
       </c>
     </row>
     <row r="14">
@@ -1002,43 +1002,615 @@
         <v>12</v>
       </c>
       <c r="B14" t="n">
+        <v>17</v>
+      </c>
+      <c r="C14" t="n">
+        <v>0.0022982</v>
+      </c>
+      <c r="D14" t="n">
+        <v>1.51</v>
+      </c>
+      <c r="E14" t="n">
+        <v>3.34</v>
+      </c>
+      <c r="F14" t="n">
+        <v>6.48</v>
+      </c>
+      <c r="G14" t="n">
+        <v>12.1</v>
+      </c>
+      <c r="H14" t="n">
+        <v>15.8</v>
+      </c>
+      <c r="I14" t="n">
+        <v>21.38</v>
+      </c>
+      <c r="J14" t="n">
+        <v>28.03</v>
+      </c>
+      <c r="K14" t="n">
+        <v>34.8</v>
+      </c>
+      <c r="L14" t="n">
+        <v>41.47</v>
+      </c>
+      <c r="M14" t="n">
+        <v>49.52</v>
+      </c>
+      <c r="N14" t="n">
+        <v>21.44</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="1" t="n">
+        <v>13</v>
+      </c>
+      <c r="B15" t="n">
+        <v>18</v>
+      </c>
+      <c r="C15" t="n">
+        <v>0.0038908</v>
+      </c>
+      <c r="D15" t="n">
+        <v>1.59</v>
+      </c>
+      <c r="E15" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="F15" t="n">
+        <v>7.32</v>
+      </c>
+      <c r="G15" t="n">
+        <v>13.64</v>
+      </c>
+      <c r="H15" t="n">
+        <v>18.35</v>
+      </c>
+      <c r="I15" t="n">
+        <v>25.2</v>
+      </c>
+      <c r="J15" t="n">
+        <v>33.41</v>
+      </c>
+      <c r="K15" t="n">
+        <v>42.11</v>
+      </c>
+      <c r="L15" t="n">
+        <v>51.21</v>
+      </c>
+      <c r="M15" t="n">
+        <v>62.07</v>
+      </c>
+      <c r="N15" t="n">
+        <v>25.86</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="1" t="n">
+        <v>14</v>
+      </c>
+      <c r="B16" t="n">
+        <v>19</v>
+      </c>
+      <c r="C16" t="n">
+        <v>0.0051222</v>
+      </c>
+      <c r="D16" t="n">
+        <v>1.63</v>
+      </c>
+      <c r="E16" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="F16" t="n">
+        <v>7.54</v>
+      </c>
+      <c r="G16" t="n">
+        <v>14</v>
+      </c>
+      <c r="H16" t="n">
+        <v>18.9</v>
+      </c>
+      <c r="I16" t="n">
+        <v>25.99</v>
+      </c>
+      <c r="J16" t="n">
+        <v>34.46</v>
+      </c>
+      <c r="K16" t="n">
+        <v>43.49</v>
+      </c>
+      <c r="L16" t="n">
+        <v>53</v>
+      </c>
+      <c r="M16" t="n">
+        <v>64.33</v>
+      </c>
+      <c r="N16" t="n">
+        <v>26.71</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="1" t="n">
+        <v>15</v>
+      </c>
+      <c r="B17" t="n">
+        <v>20</v>
+      </c>
+      <c r="C17" t="n">
+        <v>0.0068998</v>
+      </c>
+      <c r="D17" t="n">
+        <v>1.63</v>
+      </c>
+      <c r="E17" t="n">
+        <v>3.79</v>
+      </c>
+      <c r="F17" t="n">
+        <v>7.48</v>
+      </c>
+      <c r="G17" t="n">
+        <v>13.88</v>
+      </c>
+      <c r="H17" t="n">
+        <v>18.68</v>
+      </c>
+      <c r="I17" t="n">
+        <v>25.65</v>
+      </c>
+      <c r="J17" t="n">
+        <v>33.97</v>
+      </c>
+      <c r="K17" t="n">
+        <v>42.81</v>
+      </c>
+      <c r="L17" t="n">
+        <v>52.08</v>
+      </c>
+      <c r="M17" t="n">
+        <v>63.14</v>
+      </c>
+      <c r="N17" t="n">
+        <v>26.31</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="1" t="n">
+        <v>16</v>
+      </c>
+      <c r="B18" t="n">
+        <v>21</v>
+      </c>
+      <c r="C18" t="n">
+        <v>0.003561</v>
+      </c>
+      <c r="D18" t="n">
+        <v>1.66</v>
+      </c>
+      <c r="E18" t="n">
+        <v>3.96</v>
+      </c>
+      <c r="F18" t="n">
+        <v>7.93</v>
+      </c>
+      <c r="G18" t="n">
+        <v>14.73</v>
+      </c>
+      <c r="H18" t="n">
+        <v>20.12</v>
+      </c>
+      <c r="I18" t="n">
+        <v>27.83</v>
+      </c>
+      <c r="J18" t="n">
+        <v>37.05</v>
+      </c>
+      <c r="K18" t="n">
+        <v>47</v>
+      </c>
+      <c r="L18" t="n">
+        <v>57.66</v>
+      </c>
+      <c r="M18" t="n">
+        <v>70.31</v>
+      </c>
+      <c r="N18" t="n">
+        <v>28.82</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="1" t="n">
+        <v>17</v>
+      </c>
+      <c r="B19" t="n">
+        <v>22</v>
+      </c>
+      <c r="C19" t="n">
+        <v>0.038738</v>
+      </c>
+      <c r="D19" t="n">
+        <v>1.35</v>
+      </c>
+      <c r="E19" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F19" t="n">
+        <v>4.41</v>
+      </c>
+      <c r="G19" t="n">
+        <v>8.33</v>
+      </c>
+      <c r="H19" t="n">
+        <v>9.67</v>
+      </c>
+      <c r="I19" t="n">
+        <v>12.4</v>
+      </c>
+      <c r="J19" t="n">
+        <v>15.71</v>
+      </c>
+      <c r="K19" t="n">
+        <v>18.5</v>
+      </c>
+      <c r="L19" t="n">
+        <v>20.28</v>
+      </c>
+      <c r="M19" t="n">
+        <v>22.87</v>
+      </c>
+      <c r="N19" t="n">
+        <v>11.6</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="1" t="n">
+        <v>18</v>
+      </c>
+      <c r="B20" t="n">
+        <v>23</v>
+      </c>
+      <c r="C20" t="n">
+        <v>0.0051528</v>
+      </c>
+      <c r="D20" t="n">
+        <v>1.62</v>
+      </c>
+      <c r="E20" t="n">
+        <v>3.81</v>
+      </c>
+      <c r="F20" t="n">
+        <v>7.54</v>
+      </c>
+      <c r="G20" t="n">
+        <v>14.02</v>
+      </c>
+      <c r="H20" t="n">
+        <v>18.94</v>
+      </c>
+      <c r="I20" t="n">
+        <v>26.06</v>
+      </c>
+      <c r="J20" t="n">
+        <v>34.57</v>
+      </c>
+      <c r="K20" t="n">
+        <v>43.65</v>
+      </c>
+      <c r="L20" t="n">
+        <v>53.21</v>
+      </c>
+      <c r="M20" t="n">
+        <v>64.61</v>
+      </c>
+      <c r="N20" t="n">
+        <v>26.8</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="1" t="n">
+        <v>19</v>
+      </c>
+      <c r="B21" t="n">
+        <v>24</v>
+      </c>
+      <c r="C21" t="n">
+        <v>0.096053</v>
+      </c>
+      <c r="D21" t="n">
+        <v>1.39</v>
+      </c>
+      <c r="E21" t="n">
+        <v>2.62</v>
+      </c>
+      <c r="F21" t="n">
+        <v>4.66</v>
+      </c>
+      <c r="G21" t="n">
+        <v>8.74</v>
+      </c>
+      <c r="H21" t="n">
+        <v>10.31</v>
+      </c>
+      <c r="I21" t="n">
+        <v>13.31</v>
+      </c>
+      <c r="J21" t="n">
+        <v>16.93</v>
+      </c>
+      <c r="K21" t="n">
+        <v>20.09</v>
+      </c>
+      <c r="L21" t="n">
+        <v>22.31</v>
+      </c>
+      <c r="M21" t="n">
+        <v>25.4</v>
+      </c>
+      <c r="N21" t="n">
+        <v>12.58</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="1" t="n">
+        <v>20</v>
+      </c>
+      <c r="B22" t="n">
+        <v>25</v>
+      </c>
+      <c r="C22" t="n">
+        <v>0.012833</v>
+      </c>
+      <c r="D22" t="n">
+        <v>1.54</v>
+      </c>
+      <c r="E22" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="F22" t="n">
+        <v>7.19</v>
+      </c>
+      <c r="G22" t="n">
+        <v>13.49</v>
+      </c>
+      <c r="H22" t="n">
+        <v>18.19</v>
+      </c>
+      <c r="I22" t="n">
+        <v>25.06</v>
+      </c>
+      <c r="J22" t="n">
+        <v>33.29</v>
+      </c>
+      <c r="K22" t="n">
+        <v>42.03</v>
+      </c>
+      <c r="L22" t="n">
+        <v>51.2</v>
+      </c>
+      <c r="M22" t="n">
+        <v>62.15</v>
+      </c>
+      <c r="N22" t="n">
+        <v>25.78</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="1" t="n">
+        <v>21</v>
+      </c>
+      <c r="B23" t="n">
+        <v>26</v>
+      </c>
+      <c r="C23" t="n">
+        <v>0.044956</v>
+      </c>
+      <c r="D23" t="n">
+        <v>1.49</v>
+      </c>
+      <c r="E23" t="n">
+        <v>3.37</v>
+      </c>
+      <c r="F23" t="n">
+        <v>4.62</v>
+      </c>
+      <c r="G23" t="n">
+        <v>3.79</v>
+      </c>
+      <c r="H23" t="n">
+        <v>6.03</v>
+      </c>
+      <c r="I23" t="n">
+        <v>6.87</v>
+      </c>
+      <c r="J23" t="n">
+        <v>7.2</v>
+      </c>
+      <c r="K23" t="n">
+        <v>8.380000000000001</v>
+      </c>
+      <c r="L23" t="n">
+        <v>11.25</v>
+      </c>
+      <c r="M23" t="n">
+        <v>13.43</v>
+      </c>
+      <c r="N23" t="n">
+        <v>6.64</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="1" t="n">
+        <v>22</v>
+      </c>
+      <c r="B24" t="n">
+        <v>27</v>
+      </c>
+      <c r="C24" t="n">
+        <v>0.029329</v>
+      </c>
+      <c r="D24" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E24" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="F24" t="n">
+        <v>0.29</v>
+      </c>
+      <c r="G24" t="n">
+        <v>2.35</v>
+      </c>
+      <c r="H24" t="n">
+        <v>2.34</v>
+      </c>
+      <c r="I24" t="n">
+        <v>3.89</v>
+      </c>
+      <c r="J24" t="n">
+        <v>6.13</v>
+      </c>
+      <c r="K24" t="n">
+        <v>7.87</v>
+      </c>
+      <c r="L24" t="n">
+        <v>8.49</v>
+      </c>
+      <c r="M24" t="n">
+        <v>10.05</v>
+      </c>
+      <c r="N24" t="n">
+        <v>4.24</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="1" t="n">
+        <v>23</v>
+      </c>
+      <c r="B25" t="n">
+        <v>28</v>
+      </c>
+      <c r="C25" t="n">
+        <v>0.12669</v>
+      </c>
+      <c r="D25" t="n">
+        <v>1.26</v>
+      </c>
+      <c r="E25" t="n">
+        <v>1.99</v>
+      </c>
+      <c r="F25" t="n">
+        <v>3.13</v>
+      </c>
+      <c r="G25" t="n">
+        <v>5.95</v>
+      </c>
+      <c r="H25" t="n">
+        <v>5.75</v>
+      </c>
+      <c r="I25" t="n">
+        <v>6.56</v>
+      </c>
+      <c r="J25" t="n">
+        <v>7.57</v>
+      </c>
+      <c r="K25" t="n">
+        <v>7.57</v>
+      </c>
+      <c r="L25" t="n">
+        <v>5.86</v>
+      </c>
+      <c r="M25" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="N25" t="n">
+        <v>5.01</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="1" t="n">
+        <v>24</v>
+      </c>
+      <c r="B26" t="n">
+        <v>29</v>
+      </c>
+      <c r="C26" t="n">
+        <v>0.017513</v>
+      </c>
+      <c r="D26" t="n">
+        <v>1.68</v>
+      </c>
+      <c r="E26" t="n">
+        <v>3.88</v>
+      </c>
+      <c r="F26" t="n">
+        <v>7.57</v>
+      </c>
+      <c r="G26" t="n">
+        <v>13.95</v>
+      </c>
+      <c r="H26" t="n">
+        <v>18.71</v>
+      </c>
+      <c r="I26" t="n">
+        <v>25.6</v>
+      </c>
+      <c r="J26" t="n">
+        <v>33.81</v>
+      </c>
+      <c r="K26" t="n">
+        <v>42.5</v>
+      </c>
+      <c r="L26" t="n">
+        <v>51.57</v>
+      </c>
+      <c r="M26" t="n">
+        <v>62.38</v>
+      </c>
+      <c r="N26" t="n">
+        <v>26.17</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="1" t="n">
+        <v>25</v>
+      </c>
+      <c r="B27" t="n">
         <v>30</v>
       </c>
-      <c r="C14" t="n">
-        <v>0.084518</v>
-      </c>
-      <c r="D14" t="n">
-        <v>34.4</v>
-      </c>
-      <c r="E14" t="n">
-        <v>42.35</v>
-      </c>
-      <c r="F14" t="n">
-        <v>67.11</v>
-      </c>
-      <c r="G14" t="n">
-        <v>59.31</v>
-      </c>
-      <c r="H14" t="n">
-        <v>85.97</v>
-      </c>
-      <c r="I14" t="n">
-        <v>111.9</v>
-      </c>
-      <c r="J14" t="n">
-        <v>153.69</v>
-      </c>
-      <c r="K14" t="n">
-        <v>177.84</v>
-      </c>
-      <c r="L14" t="n">
-        <v>235.95</v>
-      </c>
-      <c r="M14" t="n">
-        <v>308.63</v>
-      </c>
-      <c r="N14" t="n">
-        <v>127.72</v>
+      <c r="C27" t="n">
+        <v>0.037567</v>
+      </c>
+      <c r="D27" t="n">
+        <v>1.59</v>
+      </c>
+      <c r="E27" t="n">
+        <v>3.46</v>
+      </c>
+      <c r="F27" t="n">
+        <v>6.56</v>
+      </c>
+      <c r="G27" t="n">
+        <v>12.09</v>
+      </c>
+      <c r="H27" t="n">
+        <v>15.64</v>
+      </c>
+      <c r="I27" t="n">
+        <v>21</v>
+      </c>
+      <c r="J27" t="n">
+        <v>27.36</v>
+      </c>
+      <c r="K27" t="n">
+        <v>33.78</v>
+      </c>
+      <c r="L27" t="n">
+        <v>39.99</v>
+      </c>
+      <c r="M27" t="n">
+        <v>47.51</v>
+      </c>
+      <c r="N27" t="n">
+        <v>20.9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>